<commit_message>
chore: update dashboard v2 workbook to version 5
</commit_message>
<xml_diff>
--- a/client/public/dashboard-v2.xlsx
+++ b/client/public/dashboard-v2.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/home/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9BBF37D-9E32-D749-ABD8-F29A764C6FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9788E4-BA60-CC45-B4AE-80E4653188B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18020" xr2:uid="{3A949835-928B-43F0-8F59-3C1F84CFAB50}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18160" activeTab="1" xr2:uid="{3A949835-928B-43F0-8F59-3C1F84CFAB50}"/>
   </bookViews>
   <sheets>
-    <sheet name="Template Version 2" sheetId="5" r:id="rId1"/>
-    <sheet name="Template Version 1" sheetId="1" state="hidden" r:id="rId2"/>
+    <sheet name="Change Log" sheetId="6" r:id="rId1"/>
+    <sheet name="Template Version 5" sheetId="5" r:id="rId2"/>
+    <sheet name="Template Version 1" sheetId="1" state="hidden" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="114">
   <si>
     <t>Day</t>
   </si>
@@ -348,9 +349,6 @@
     <t>CM 2 Due On</t>
   </si>
   <si>
-    <t>00/00/00</t>
-  </si>
-  <si>
     <t>Available</t>
   </si>
   <si>
@@ -360,18 +358,43 @@
     <t>Remaining AFTER Attack</t>
   </si>
   <si>
-    <t>1/0/1900</t>
+    <t>Quick Note: https://buymeacoffee.com/theultimatejourney</t>
+  </si>
+  <si>
+    <t>00/00/0000</t>
+  </si>
+  <si>
+    <t>Days Left:</t>
+  </si>
+  <si>
+    <t>Latest Due By Date</t>
+  </si>
+  <si>
+    <t>Change Requested By</t>
+  </si>
+  <si>
+    <t>Assigned To</t>
+  </si>
+  <si>
+    <t>Request</t>
+  </si>
+  <si>
+    <t>BSA Note</t>
+  </si>
+  <si>
+    <t>Completion Date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     <numFmt numFmtId="165" formatCode="mmm\-yyyy"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,6 +440,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF92D050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -496,7 +527,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -582,12 +613,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -805,21 +851,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -830,8 +861,86 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1147,12 +1256,46 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E79790A0-8B41-F94C-92A1-BAEDBA4D0CB1}">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="116" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="116" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" s="116" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="116" t="s">
+        <v>111</v>
+      </c>
+      <c r="E1" s="116" t="s">
+        <v>112</v>
+      </c>
+      <c r="F1" s="116" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE1543BC-89E0-46D1-A050-F10A0CF8D26C}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:W51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="43.5" customWidth="1"/>
+    <col min="1" max="1" width="47" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
@@ -1177,7 +1320,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="92"/>
+      <c r="A1" s="115"/>
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -1204,27 +1347,29 @@
       </c>
     </row>
     <row r="2" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="92"/>
+      <c r="A2" s="115"/>
       <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
       <c r="D2" s="5">
         <v>0</v>
       </c>
-      <c r="E2" s="9">
-        <v>0</v>
-      </c>
-      <c r="F2" s="7">
-        <v>0</v>
-      </c>
-      <c r="G2" s="8">
+      <c r="E2" s="89">
+        <v>0</v>
+      </c>
+      <c r="F2" s="90">
+        <v>0</v>
+      </c>
+      <c r="G2" s="92">
         <f>D3</f>
         <v>0</v>
       </c>
-      <c r="H2" s="6">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6">
-        <f>E2+G2</f>
+      <c r="H2" s="91">
+        <v>0</v>
+      </c>
+      <c r="I2" s="91">
+        <f>B13+B14</f>
         <v>0</v>
       </c>
       <c r="J2" s="9"/>
@@ -1236,27 +1381,27 @@
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:17" ht="33" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
+      <c r="A3" s="115"/>
       <c r="B3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="93">
         <f>IF(J23&gt;L23,D3,D3-(L23-J23)+G17)</f>
         <v>0</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="95">
         <v>0</v>
       </c>
       <c r="E3" s="3"/>
-      <c r="F3" s="6">
+      <c r="F3" s="91">
         <f>-F2+500</f>
         <v>500</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="91">
         <f>E2</f>
         <v>0</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="91">
         <f>F2+C9</f>
         <v>0</v>
       </c>
@@ -1265,37 +1410,37 @@
       </c>
       <c r="K3" s="14"/>
       <c r="Q3" s="2" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="92"/>
+      <c r="A4" s="115"/>
       <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="91">
         <f>D25+D26</f>
         <v>0</v>
       </c>
-      <c r="D4" s="22">
-        <v>0</v>
-      </c>
-      <c r="E4" s="27" t="s">
+      <c r="D4" s="96" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="97" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="114">
         <f>F3+F2</f>
         <v>500</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="114">
         <f>G2+G3</f>
         <v>0</v>
       </c>
-      <c r="I4" s="17">
+      <c r="I4" s="112">
         <f>SUM(I2:I3)</f>
         <v>0</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="111">
         <f>B12+I4+G17</f>
         <v>0</v>
       </c>
@@ -1314,24 +1459,23 @@
       <c r="P4" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="Q4" s="14">
-        <f>H$13</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="92"/>
+      <c r="Q4" s="29" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="19" x14ac:dyDescent="0.25">
+      <c r="A5" s="115"/>
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="91">
         <f>SUM(D5:E5)-E11</f>
         <v>0</v>
       </c>
-      <c r="D5" s="22">
-        <v>0</v>
-      </c>
-      <c r="E5" s="24">
+      <c r="D5" s="96">
+        <v>0</v>
+      </c>
+      <c r="E5" s="98">
         <v>0</v>
       </c>
       <c r="F5" s="10" t="s">
@@ -1348,17 +1492,20 @@
       <c r="O5" s="10">
         <v>-7500</v>
       </c>
-      <c r="P5" s="26" t="str">
-        <f>IF(J$4&lt;O5, "&lt;", "")</f>
-        <v/>
+      <c r="P5" s="45" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q5" s="88" t="e">
+        <f ca="1">MAX(0,Q4-TODAY())</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="92"/>
+      <c r="A6" s="115"/>
       <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="91">
         <f>D27</f>
         <v>0</v>
       </c>
@@ -1387,11 +1534,11 @@
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="92"/>
+      <c r="A7" s="115"/>
       <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="91">
         <f t="shared" ref="C7:C8" si="3">D28</f>
         <v>0</v>
       </c>
@@ -1421,11 +1568,11 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="92"/>
+      <c r="A8" s="115"/>
       <c r="B8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="91">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1455,11 +1602,11 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="92"/>
+      <c r="A9" s="115"/>
       <c r="B9" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="81">
+      <c r="C9" s="94">
         <f>SUM(D9:E9)</f>
         <v>0</v>
       </c>
@@ -1492,7 +1639,7 @@
       <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="91">
         <f>C3</f>
         <v>0</v>
       </c>
@@ -1518,10 +1665,10 @@
     </row>
     <row r="11" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>105</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C11" s="28" t="str">
         <f>IF(B13&gt;0,"There is a CM Approaching","All Clear")</f>
@@ -1530,12 +1677,12 @@
       <c r="D11" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="89">
         <f>F6+F7+F8+F9</f>
         <v>0</v>
       </c>
-      <c r="H11" s="29">
-        <v>0</v>
+      <c r="H11" s="29" t="s">
+        <v>106</v>
       </c>
       <c r="M11" s="19" t="str">
         <f t="shared" si="0"/>
@@ -1569,7 +1716,7 @@
         <v>31</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>33</v>
@@ -1607,42 +1754,42 @@
       <c r="A13" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="22">
-        <v>0</v>
-      </c>
-      <c r="C13" s="35">
-        <v>0</v>
-      </c>
-      <c r="D13" s="22">
+      <c r="B13" s="96">
+        <v>0</v>
+      </c>
+      <c r="C13" s="99">
+        <v>0</v>
+      </c>
+      <c r="D13" s="96">
         <f>B13-C13</f>
         <v>0</v>
       </c>
-      <c r="E13" s="36">
+      <c r="E13" s="100">
         <f>I13</f>
         <v>0</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="96">
         <f>B13-E13</f>
         <v>0</v>
       </c>
-      <c r="G13" s="37">
-        <f>H13-C2</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="38">
-        <v>0</v>
-      </c>
-      <c r="I13" s="22">
-        <v>0</v>
-      </c>
-      <c r="J13" s="24">
+      <c r="G13" s="37" t="str">
+        <f>IFERROR(IF(OR(H13=0,C2=0),"",H13-C2),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="I13" s="96">
+        <v>0</v>
+      </c>
+      <c r="J13" s="98">
         <f>L13</f>
         <v>0</v>
       </c>
       <c r="K13" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L13" s="22">
+      <c r="L13" s="96">
         <f>C13</f>
         <v>0</v>
       </c>
@@ -1664,42 +1811,42 @@
       <c r="A14" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="22">
-        <v>0</v>
-      </c>
-      <c r="C14" s="35">
-        <v>0</v>
-      </c>
-      <c r="D14" s="22">
+      <c r="B14" s="96">
+        <v>0</v>
+      </c>
+      <c r="C14" s="99">
+        <v>0</v>
+      </c>
+      <c r="D14" s="96">
         <f>B14-C14</f>
         <v>0</v>
       </c>
-      <c r="E14" s="36">
+      <c r="E14" s="100">
         <f>I14</f>
         <v>0</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="96">
         <f>B14-E14</f>
         <v>0</v>
       </c>
-      <c r="G14" s="37" t="e">
-        <f>H14-C2</f>
-        <v>#VALUE!</v>
+      <c r="G14" s="37" t="str">
+        <f>IFERROR(IF(OR(H14=0,C2=0),"",H14-C2),"")</f>
+        <v/>
       </c>
       <c r="H14" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="I14" s="22">
-        <v>0</v>
-      </c>
-      <c r="J14" s="24">
+      <c r="I14" s="96">
+        <v>0</v>
+      </c>
+      <c r="J14" s="98">
         <f>L14</f>
         <v>0</v>
       </c>
       <c r="K14" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L14" s="22">
+      <c r="L14" s="96">
         <f>C14</f>
         <v>0</v>
       </c>
@@ -1721,23 +1868,23 @@
       <c r="A15" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="58">
+      <c r="B15" s="93">
         <f>SUM(B13:B14)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="35">
+      <c r="C15" s="99">
         <f>SUM(C13:C14)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="96">
         <f>SUM(D13:D14)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="100">
         <f>SUM(E13:E14)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="40">
+      <c r="F15" s="101">
         <f>SUM(F13:F14)</f>
         <v>0</v>
       </c>
@@ -1745,18 +1892,18 @@
       <c r="H15" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="I15" s="41">
+      <c r="I15" s="102">
         <f>SUM(I13:I14)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="24">
+      <c r="J15" s="98">
         <f>SUM(J13:J14)</f>
         <v>0</v>
       </c>
       <c r="K15" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L15" s="22">
+      <c r="L15" s="96">
         <f>SUM(L13:L14)</f>
         <v>0</v>
       </c>
@@ -1800,7 +1947,7 @@
       <c r="A17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="46">
+      <c r="B17" s="103">
         <v>0</v>
       </c>
       <c r="C17" s="10" t="s">
@@ -1832,14 +1979,14 @@
       <c r="A18">
         <v>1</v>
       </c>
-      <c r="B18" s="46">
+      <c r="B18" s="103">
         <v>0</v>
       </c>
       <c r="C18" s="15" t="str">
         <f>IF(B28&gt;B17,"Increase","Decrease")</f>
         <v>Decrease</v>
       </c>
-      <c r="D18" s="51">
+      <c r="D18" s="105">
         <f>B28-B17</f>
         <v>0</v>
       </c>
@@ -1867,16 +2014,16 @@
       <c r="A19">
         <v>2</v>
       </c>
-      <c r="B19" s="46">
+      <c r="B19" s="103">
         <v>0</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="52">
+      <c r="F19" s="52" t="str">
         <f>H11</f>
-        <v>0</v>
+        <v>00/00/0000</v>
       </c>
       <c r="G19" s="10"/>
       <c r="H19" s="15" t="s">
@@ -1888,9 +2035,9 @@
       <c r="K19" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="L19" s="53">
+      <c r="L19" s="53" t="str">
         <f>H13</f>
-        <v>0</v>
+        <v>00/00/0000</v>
       </c>
       <c r="M19" s="19" t="str">
         <f t="shared" si="0"/>
@@ -1910,7 +2057,7 @@
       <c r="A20">
         <v>3</v>
       </c>
-      <c r="B20" s="46">
+      <c r="B20" s="96">
         <v>0</v>
       </c>
       <c r="D20" s="10"/>
@@ -1927,15 +2074,15 @@
       <c r="I20" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="J20" s="57">
-        <f>I15</f>
+      <c r="J20" s="104">
+        <f>J15</f>
         <v>0</v>
       </c>
       <c r="K20" s="54" t="str">
         <f>IF(J20 &gt;=L20, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L20" s="58">
+      <c r="L20" s="93">
         <f>L15</f>
         <v>0</v>
       </c>
@@ -1957,26 +2104,26 @@
       <c r="A21">
         <v>4</v>
       </c>
-      <c r="B21" s="46">
+      <c r="B21" s="96">
         <v>0</v>
       </c>
       <c r="D21" s="10"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="59">
+      <c r="F21" s="59" t="str">
         <f>H13</f>
-        <v>0</v>
-      </c>
-      <c r="G21" s="82">
-        <f>F21-E23</f>
-        <v>0</v>
-      </c>
-      <c r="H21" s="88" t="s">
+        <v>00/00/0000</v>
+      </c>
+      <c r="G21" s="82" t="str">
+        <f>IFERROR(IF(OR(F21=0,E23=0),"",F21-E23),"")</f>
+        <v/>
+      </c>
+      <c r="H21" s="83" t="s">
         <v>98</v>
       </c>
       <c r="I21" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="J21" s="58">
+      <c r="J21" s="93">
         <f>D25</f>
         <v>0</v>
       </c>
@@ -1984,7 +2131,7 @@
         <f>IF(J21 =L21, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L21" s="58">
+      <c r="L21" s="93">
         <f>D25</f>
         <v>0</v>
       </c>
@@ -2006,7 +2153,8 @@
       <c r="A22">
         <v>5</v>
       </c>
-      <c r="B22" s="46">
+      <c r="B22" s="96">
+        <f t="shared" ref="B22" si="4">SUM(B17:B21)</f>
         <v>0</v>
       </c>
       <c r="D22" s="10"/>
@@ -2023,7 +2171,7 @@
       <c r="I22" s="56" t="s">
         <v>60</v>
       </c>
-      <c r="J22" s="57">
+      <c r="J22" s="104">
         <f>D26</f>
         <v>0</v>
       </c>
@@ -2031,7 +2179,7 @@
         <f>IF(J22 =L22, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L22" s="58">
+      <c r="L22" s="93">
         <f>D26</f>
         <v>0</v>
       </c>
@@ -2053,7 +2201,7 @@
       <c r="A23">
         <v>6</v>
       </c>
-      <c r="B23" s="46">
+      <c r="B23" s="103">
         <v>0</v>
       </c>
       <c r="D23" s="10"/>
@@ -2061,20 +2209,21 @@
         <f>C2</f>
         <v>0</v>
       </c>
-      <c r="F23" s="61" t="s">
+      <c r="F23" s="61" t="str">
+        <f>H14</f>
+        <v>00/00/0000</v>
+      </c>
+      <c r="G23" s="82" t="str">
+        <f>IFERROR(IF(OR(F23=0,E23=0),"",F23-E23),"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="83" t="s">
+        <v>97</v>
+      </c>
+      <c r="I23" s="58" t="s">
         <v>102</v>
       </c>
-      <c r="G23" s="82" t="e">
-        <f>IMSUB(F23,E23)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="H23" s="88" t="s">
-        <v>97</v>
-      </c>
-      <c r="I23" s="58" t="s">
-        <v>103</v>
-      </c>
-      <c r="J23" s="18">
+      <c r="J23" s="111">
         <f>SUM(J20:J22)</f>
         <v>0</v>
       </c>
@@ -2082,7 +2231,7 @@
         <f>IF(J23 =L23, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L23" s="58">
+      <c r="L23" s="93">
         <f>SUM(L20:L22)</f>
         <v>0</v>
       </c>
@@ -2104,7 +2253,7 @@
       <c r="A24">
         <v>7</v>
       </c>
-      <c r="B24" s="46">
+      <c r="B24" s="103">
         <v>0</v>
       </c>
       <c r="C24" s="15" t="s">
@@ -2114,12 +2263,12 @@
       <c r="E24" s="62" t="s">
         <v>99</v>
       </c>
-      <c r="G24" s="89"/>
-      <c r="H24" s="89"/>
-      <c r="I24" s="90"/>
-      <c r="J24" s="91"/>
+      <c r="G24" s="84"/>
+      <c r="H24" s="84"/>
+      <c r="I24" s="85"/>
+      <c r="J24" s="86"/>
       <c r="K24" s="72"/>
-      <c r="L24" s="89"/>
+      <c r="L24" s="84"/>
       <c r="M24" s="19" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2138,24 +2287,24 @@
       <c r="A25">
         <v>8</v>
       </c>
-      <c r="B25" s="46">
+      <c r="B25" s="103">
         <v>0</v>
       </c>
       <c r="C25" s="2" t="str">
         <f>I21</f>
         <v>Mortgage</v>
       </c>
-      <c r="D25" s="62">
-        <v>0</v>
-      </c>
-      <c r="E25" s="4">
+      <c r="D25" s="103">
+        <v>0</v>
+      </c>
+      <c r="E25" s="87">
         <f>C$2</f>
         <v>0</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="83">
+      <c r="H25" s="106">
         <f>F2</f>
         <v>0</v>
       </c>
@@ -2189,33 +2338,33 @@
       <c r="A26">
         <v>9</v>
       </c>
-      <c r="B26" s="46">
+      <c r="B26" s="96">
         <v>0</v>
       </c>
       <c r="C26" s="2" t="str">
         <f>I22</f>
         <v>HOA</v>
       </c>
-      <c r="D26" s="62">
-        <v>0</v>
-      </c>
-      <c r="E26" s="4">
-        <f t="shared" ref="E26:E29" si="4">C$2</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="84">
+      <c r="D26" s="103">
+        <v>0</v>
+      </c>
+      <c r="E26" s="87">
+        <f t="shared" ref="E26:E29" si="5">C$2</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="107">
         <f>G2</f>
         <v>0</v>
       </c>
-      <c r="I26" s="66">
+      <c r="I26" s="98">
         <f>G17+C3+F2-I15-M50+E11</f>
         <v>0</v>
       </c>
-      <c r="J26" s="66">
+      <c r="J26" s="98">
         <f>G17+C3+C8+F2-M50</f>
         <v>0</v>
       </c>
-      <c r="K26" s="67">
+      <c r="K26" s="113">
         <v>5000</v>
       </c>
       <c r="L26" s="68" t="str">
@@ -2240,24 +2389,24 @@
       <c r="A27">
         <v>10</v>
       </c>
-      <c r="B27" s="46">
+      <c r="B27" s="96">
         <v>0</v>
       </c>
       <c r="C27" s="2" t="str">
         <f>B6</f>
         <v>Vacation Savings</v>
       </c>
-      <c r="D27" s="62">
-        <v>0</v>
-      </c>
-      <c r="E27" s="4">
-        <f t="shared" si="4"/>
+      <c r="D27" s="103">
+        <v>0</v>
+      </c>
+      <c r="E27" s="87">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G27" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="H27" s="85">
+      <c r="H27" s="108">
         <f>SUM(H25:H26)</f>
         <v>0</v>
       </c>
@@ -2283,24 +2432,25 @@
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="46">
+      <c r="B28" s="96">
+        <f t="shared" ref="B28" si="6">SUM(B23:B27)</f>
         <v>0</v>
       </c>
       <c r="C28" s="2" t="str">
         <f>B7</f>
         <v>Emergency Savings</v>
       </c>
-      <c r="D28" s="22">
-        <v>0</v>
-      </c>
-      <c r="E28" s="4">
-        <f t="shared" si="4"/>
+      <c r="D28" s="96">
+        <v>0</v>
+      </c>
+      <c r="E28" s="87">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="H28" s="86">
+      <c r="H28" s="109">
         <f>H27-D30</f>
         <v>0</v>
       </c>
@@ -2329,17 +2479,17 @@
         <f>B8</f>
         <v>Boost Savings</v>
       </c>
-      <c r="D29" s="22">
-        <v>0</v>
-      </c>
-      <c r="E29" s="4">
-        <f t="shared" si="4"/>
+      <c r="D29" s="96">
+        <v>0</v>
+      </c>
+      <c r="E29" s="87">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G29" t="s">
         <v>71</v>
       </c>
-      <c r="H29" s="87">
+      <c r="H29" s="110">
         <f>H27+G17</f>
         <v>0</v>
       </c>
@@ -2362,10 +2512,11 @@
       <c r="Q29" s="30"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="B30" s="117"/>
       <c r="C30" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="22">
+      <c r="D30" s="96">
         <f>SUM(D25:D29)</f>
         <v>0</v>
       </c>
@@ -2389,6 +2540,7 @@
       <c r="Q30" s="30"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="B31" s="22"/>
       <c r="C31" s="2"/>
       <c r="D31" s="10"/>
       <c r="H31" s="10"/>
@@ -2403,6 +2555,7 @@
       <c r="Q31" s="10"/>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="B32" s="6"/>
       <c r="H32" s="10"/>
       <c r="I32" s="10"/>
       <c r="J32" s="13"/>
@@ -2415,31 +2568,17 @@
       <c r="Q32" s="10"/>
       <c r="W32" s="10"/>
     </row>
-    <row r="33" spans="1:20" ht="32" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:20" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="E33" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F33" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="G33" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="H33" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="I33" s="27" t="s">
-        <v>79</v>
-      </c>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27"/>
       <c r="J33" s="15"/>
       <c r="K33" s="15" t="s">
         <v>80</v>
@@ -2479,20 +2618,20 @@
       <c r="L34" s="72"/>
       <c r="M34" s="69"/>
       <c r="N34" s="74">
-        <f>I26</f>
-        <v>0</v>
-      </c>
-      <c r="O34" s="37" t="e">
-        <f>N34/Q50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P34" s="37" t="e">
-        <f>O34/Q50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q34" s="37" t="e">
-        <f>P34/Q50</f>
-        <v>#DIV/0!</v>
+        <f>IFERROR(I26,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O34" s="37">
+        <f>IFERROR(N34/Q50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P34" s="37">
+        <f>IFERROR(O34/Q50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q34" s="37">
+        <f>IFERROR(P34/Q50,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.2">
@@ -2513,25 +2652,25 @@
       <c r="J35" s="76"/>
       <c r="K35" s="76"/>
       <c r="L35" s="76"/>
-      <c r="M35" s="57">
-        <f t="shared" ref="M35" si="5">SUM(C35:I35)</f>
+      <c r="M35" s="104">
+        <f t="shared" ref="M35" si="7">SUM(C35:I35)</f>
         <v>0</v>
       </c>
       <c r="N35" s="77">
-        <f>N34-M35</f>
-        <v>0</v>
-      </c>
-      <c r="O35" s="77" t="e">
-        <f>O34-M35/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P35" s="77" t="e">
-        <f>P34-M35/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q35" s="77" t="e">
-        <f>Q34-M35/Q$50</f>
-        <v>#DIV/0!</v>
+        <f>IFERROR(N34-M35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O35" s="77">
+        <f t="shared" ref="O35:O48" si="8">IFERROR(O34-M35/Q$50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P35" s="77">
+        <f t="shared" ref="P35:P48" si="9">IFERROR(P34-M35/Q$50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q35" s="77">
+        <f t="shared" ref="Q35:Q48" si="10">IFERROR(Q34-M35/Q$50,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.2">
@@ -2552,25 +2691,25 @@
       <c r="J36" s="76"/>
       <c r="K36" s="76"/>
       <c r="L36" s="76"/>
-      <c r="M36" s="57">
+      <c r="M36" s="104">
         <f>SUM(C36:L36)</f>
         <v>0</v>
       </c>
-      <c r="N36" s="77" t="e">
-        <f>N35-M36/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O36" s="77" t="e">
-        <f t="shared" ref="O36:O48" si="6">O35-M36/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P36" s="77" t="e">
-        <f t="shared" ref="P36:P48" si="7">P35-M36/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q36" s="77" t="e">
-        <f t="shared" ref="Q36:Q48" si="8">Q35-M36/Q$50</f>
-        <v>#DIV/0!</v>
+      <c r="N36" s="77">
+        <f t="shared" ref="N36:N48" si="11">IFERROR(N35-M36/Q$50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O36" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P36" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q36" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.2">
@@ -2591,25 +2730,25 @@
       <c r="J37" s="76"/>
       <c r="K37" s="76"/>
       <c r="L37" s="76"/>
-      <c r="M37" s="57">
+      <c r="M37" s="104">
         <f>SUM(C37:L37)</f>
         <v>0</v>
       </c>
-      <c r="N37" s="77" t="e">
-        <f t="shared" ref="N37:N48" si="9">N36-M37/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O37" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P37" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q37" s="77" t="e">
+      <c r="N37" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O37" s="77">
         <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="P37" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q37" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.2">
@@ -2630,25 +2769,25 @@
       <c r="J38" s="76"/>
       <c r="K38" s="76"/>
       <c r="L38" s="76"/>
-      <c r="M38" s="57">
-        <f t="shared" ref="M38:M48" si="10">SUM(C38:L38)</f>
-        <v>0</v>
-      </c>
-      <c r="N38" s="77" t="e">
+      <c r="M38" s="104">
+        <f t="shared" ref="M38:M48" si="12">SUM(C38:L38)</f>
+        <v>0</v>
+      </c>
+      <c r="N38" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O38" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P38" s="77">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O38" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P38" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q38" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="Q38" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.2">
@@ -2669,25 +2808,25 @@
       <c r="J39" s="76"/>
       <c r="K39" s="76"/>
       <c r="L39" s="76"/>
-      <c r="M39" s="57">
+      <c r="M39" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N39" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O39" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P39" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q39" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N39" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O39" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P39" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q39" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="40" spans="1:20" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2708,25 +2847,25 @@
       <c r="J40" s="76"/>
       <c r="K40" s="76"/>
       <c r="L40" s="76"/>
-      <c r="M40" s="57">
+      <c r="M40" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N40" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O40" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P40" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q40" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N40" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O40" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P40" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q40" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="41" spans="1:20" ht="12" customHeight="1" x14ac:dyDescent="0.2">
@@ -2747,25 +2886,25 @@
       <c r="J41" s="76"/>
       <c r="K41" s="76"/>
       <c r="L41" s="76"/>
-      <c r="M41" s="57">
+      <c r="M41" s="104">
         <f>SUM(C41:L41)</f>
         <v>0</v>
       </c>
-      <c r="N41" s="77" t="e">
+      <c r="N41" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O41" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P41" s="77">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O41" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P41" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q41" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="Q41" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.2">
@@ -2786,25 +2925,25 @@
       <c r="J42" s="76"/>
       <c r="K42" s="76"/>
       <c r="L42" s="76"/>
-      <c r="M42" s="57">
+      <c r="M42" s="104">
         <f>SUM(C42:L42)</f>
         <v>0</v>
       </c>
-      <c r="N42" s="77" t="e">
+      <c r="N42" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O42" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P42" s="77">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O42" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P42" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q42" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="Q42" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.2">
@@ -2825,25 +2964,25 @@
       <c r="J43" s="76"/>
       <c r="K43" s="76"/>
       <c r="L43" s="76"/>
-      <c r="M43" s="57">
+      <c r="M43" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N43" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O43" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P43" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q43" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N43" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O43" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P43" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q43" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.2">
@@ -2864,25 +3003,25 @@
       <c r="J44" s="76"/>
       <c r="K44" s="76"/>
       <c r="L44" s="76"/>
-      <c r="M44" s="57">
+      <c r="M44" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N44" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O44" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P44" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q44" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N44" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O44" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P44" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q44" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.2">
@@ -2903,25 +3042,25 @@
       <c r="J45" s="76"/>
       <c r="K45" s="76"/>
       <c r="L45" s="76"/>
-      <c r="M45" s="57">
+      <c r="M45" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N45" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O45" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P45" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q45" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N45" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O45" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P45" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q45" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.2">
@@ -2942,25 +3081,25 @@
       <c r="J46" s="76"/>
       <c r="K46" s="76"/>
       <c r="L46" s="76"/>
-      <c r="M46" s="57">
+      <c r="M46" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N46" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O46" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P46" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q46" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N46" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O46" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P46" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q46" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.2">
@@ -2981,25 +3120,25 @@
       <c r="J47" s="76"/>
       <c r="K47" s="76"/>
       <c r="L47" s="76"/>
-      <c r="M47" s="57">
+      <c r="M47" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N47" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O47" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P47" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q47" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N47" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O47" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P47" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q47" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.2">
@@ -3020,25 +3159,25 @@
       <c r="J48" s="78"/>
       <c r="K48" s="78"/>
       <c r="L48" s="78"/>
-      <c r="M48" s="57">
+      <c r="M48" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N48" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O48" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P48" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q48" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N48" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O48" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P48" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q48" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="49" spans="2:17" x14ac:dyDescent="0.2">
@@ -3071,61 +3210,61 @@
       <c r="B50" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C50" s="62">
+      <c r="C50" s="103">
         <f>SUM(C35:C48)</f>
         <v>0</v>
       </c>
-      <c r="D50" s="62">
+      <c r="D50" s="103">
         <f>SUM(D35:D48)</f>
         <v>0</v>
       </c>
-      <c r="E50" s="62">
-        <f t="shared" ref="E50:L50" si="11">SUM(E36:E48)</f>
-        <v>0</v>
-      </c>
-      <c r="F50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="G50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="H50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="K50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="L50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="M50" s="62">
+      <c r="E50" s="103">
+        <f t="shared" ref="E50:L50" si="13">SUM(E36:E48)</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="H50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="I50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="K50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="L50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="M50" s="103">
         <f>SUM(M35:M48)</f>
         <v>0</v>
       </c>
-      <c r="N50" s="80" t="e">
-        <f>I26/H27</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O50" s="37" t="e">
-        <f>(N34-M50)/Q50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P50" s="80" t="e">
-        <f>100% -N50</f>
-        <v>#DIV/0!</v>
+      <c r="N50" s="80">
+        <f>IFERROR(I26/H27,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O50" s="37">
+        <f>IFERROR((N34-M50)/Q50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P50" s="80">
+        <f>IFERROR(100% -N50,0)</f>
+        <v>1</v>
       </c>
       <c r="Q50" s="15">
         <f>G19</f>
@@ -3139,11 +3278,200 @@
   <mergeCells count="1">
     <mergeCell ref="A1:A9"/>
   </mergeCells>
+  <dataValidations count="47">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{3170D0ED-69B8-2147-B2E8-C845548A1AEB}">
+      <formula1>"Monday,Tuesday,Wednesday,Thursday,Friday,Saturday,Sunday"</formula1>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="Date Entry" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="C2" xr:uid="{1A0AC821-D2F1-CC47-BCD2-867E6217E64D}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Time" error="Please enter a valid time format (e.g., 11:22 AM, 14:30)" promptTitle="Time Entry" prompt="Please enter a valid time (e.g., 11:22 AM, 14:30, 8:08:00 AM)" sqref="D2" xr:uid="{725F1B26-DEA2-2544-B362-19E809BAA3B2}">
+      <formula1>0</formula1>
+      <formula2>0.999988425925926</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount (numbers only, e.g., 100.00)" promptTitle="Saved Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="E2" xr:uid="{554C6FD8-DF46-C24A-B6DA-75188B87833F}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount (numbers only)." promptTitle="Fuel Amount" prompt="Please enter a dollar amount for fuel (e.g., 50.00, 125.75)" sqref="F2" xr:uid="{2945CFF3-B39B-6B4D-A81C-A094F8872C7D}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount (number between 0 and 999,999,999.99)" promptTitle="Bank Saved Amount" prompt="Please enter a dollar amount for bank savings (e.g., 100.00, 250.50)" sqref="H2" xr:uid="{DEBEAC84-DA60-D443-A7D6-80BC8F319DBE}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="This cell contains a formula. Please edit E2 or G2 instead." promptTitle="Total Credit Card" prompt="This cell calculates the total credit card amount (Saved + Bank)" sqref="I2" xr:uid="{827C1756-1326-E340-9238-09B695E4E03F}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format (e.g., 5/15/2026)" promptTitle="Estimated Pay Drop Date" prompt="Please enter a valid date (e.g., 5/15/2026)" sqref="H11" xr:uid="{C44A92CA-E0FA-D342-848B-7ED51D8B7AC0}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format (e.g., 5/15/2026)" promptTitle="CM1 Final Due Date" prompt="Please enter a valid date (e.g., 5/15/2026)" sqref="H13 Q4" xr:uid="{9EAB60B5-5BA8-BE43-A9E2-5E5AD8961415}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format (e.g., 5/15/2026)" promptTitle="CM2 Final Due Date" prompt="Please enter a valid date (e.g., 5/15/2026)" sqref="H14" xr:uid="{0B4F1CA8-E9A3-5D46-B4E6-DCA330C9E728}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="As-Of Date (Mortgage)" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E25" xr:uid="{7F9B15EE-805C-624E-91F2-9EE5908FEB8A}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="As-Of Date (Boost Savings)" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E29" xr:uid="{9F0D187E-AECB-354E-B9D0-BBAA1D17C71F}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="Predicted Pay Drop Date" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="F19" xr:uid="{445E3649-2EF6-1244-A502-5986D5BA3DC7}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="CM 1 Due On" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="F21" xr:uid="{F6374D57-9877-D84B-A7A4-1D340524520C}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="CM 2 Due On" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="F23" xr:uid="{20D8721C-CF38-E64D-8EFB-354FA49959E5}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Bank Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="G2" xr:uid="{092CE826-655A-6846-8640-3ECBD514D949}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="HOA As-Of Date" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E26" xr:uid="{D88F751C-C1C5-1447-B3FC-0DDF32987D38}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="Vacation Savings As-Of Date" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E27" xr:uid="{2B6E4F52-F607-7849-AEE9-FBE9DE40A560}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="Emergency Savings As-Of Date" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E28" xr:uid="{4F21D987-6066-9943-B4CE-1CE92B09D0EE}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Savings Balance" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="C3:C10" xr:uid="{04DC61CC-20BC-7C47-91BB-CF0E0D2EFBA0}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Power Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D3:D5" xr:uid="{E33DAC1B-DC8C-ED4F-A043-40499074E2DF}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Water Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="E4:E5" xr:uid="{6385CA2A-90F8-BF4F-8726-40FB3E8083C6}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Debt Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="B13:B15" xr:uid="{351E97BA-1885-6540-90E2-0E2556D5428F}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Minimum Payment" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="C13:C15" xr:uid="{771F17F6-5CF3-764E-B272-86B3732C43A6}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Left 2 Go" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D13:D15" xr:uid="{AE461F65-120C-C345-8459-89C9BB09BD41}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Next Attack Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="E13:E15" xr:uid="{0069F0C6-E4A6-D14E-AFBF-52C7887ACD3B}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Remaining After Attack" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="F13:F15" xr:uid="{E60786F5-4666-3644-817A-044B60A0FD44}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Payment Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="I13:I15" xr:uid="{6BAC151E-A408-FC45-827B-DA5F226CA5FE}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Last Statement Balance" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J13:J15" xr:uid="{7B5C52C0-D156-EE4A-B1C3-2B3D6CF86CAE}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Next Minimum" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="L13:L15" xr:uid="{286008C8-7A35-FE44-875D-137AB7724D6D}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Tank Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D25:D29 B17:B21 B23:B27" xr:uid="{DCEE984F-F387-8F43-B4D2-7C222E9FA32E}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Monthly Minimum" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J20:J22" xr:uid="{32B0A9CD-D726-F24B-90D9-1712FC70AB38}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="2 Week Spending" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="M35:M48" xr:uid="{F6775EA3-3841-964B-A2C9-51770973A55B}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Holding Tank" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="E11" xr:uid="{E15B848F-7BE5-AD4D-8EA3-DF0181E63A81}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Decrease Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D18" xr:uid="{503BA0B3-FC97-E342-B416-C46429D9BB19}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Total Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="H25:H29" xr:uid="{4C020DF3-0044-6B4E-B44E-AA614A3D44BD}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Tank Total" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D30 B22 B28" xr:uid="{EB99C4F6-A363-7C40-A9E9-F2C68CD7797D}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="CM Total After Full Attack" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J4" xr:uid="{0A6AAE44-CEA8-144B-AB2F-07206831F561}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="I3:I4 G3:G4" xr:uid="{3434CA11-B4B5-F842-9DEE-B9AE2C83E338}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Current POR" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="I26" xr:uid="{79DBCC11-2E7B-524E-ADB7-9AF1D52645FD}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="All In POR" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J26" xr:uid="{CF78B612-016B-DE4B-BF60-EDF66C5A6429}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Target All-In POR (ROI)" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="K26" xr:uid="{5EDB90BD-F221-AA43-9557-DB7F094BD568}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Status Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="L20:L22" xr:uid="{BA49962A-ED1A-484B-90D9-11DC115BAE55}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Available Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J23" xr:uid="{E948AC32-8BDA-A247-9194-E7061DA8AB0E}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Monthly Minimum Status" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="L23" xr:uid="{156268F1-6A8C-7041-8A11-92E156C7B41F}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Total" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="C50:M50" xr:uid="{9DFD7696-0A1F-9044-B603-6D89D6ED2136}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Use Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="F3:F4" xr:uid="{416CBC7D-C44C-DD46-BE90-9D72426DF971}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8812D7F7-4E2E-4C59-8640-33FA123A4EE8}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:W51"/>

</xml_diff>

<commit_message>
Update dashboard workbook to Version 5
Replaces client/public/dashboard-v2.xlsx with TheUltimateJourneyDashboard-Version5.xlsx. Validated with STRIPE_SECRET_KEY=sk_test_dummy pnpm test and STRIPE_SECRET_KEY=sk_test_dummy pnpm check.
</commit_message>
<xml_diff>
--- a/client/public/dashboard-v2.xlsx
+++ b/client/public/dashboard-v2.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/home/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9BBF37D-9E32-D749-ABD8-F29A764C6FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9788E4-BA60-CC45-B4AE-80E4653188B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18020" xr2:uid="{3A949835-928B-43F0-8F59-3C1F84CFAB50}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18160" activeTab="1" xr2:uid="{3A949835-928B-43F0-8F59-3C1F84CFAB50}"/>
   </bookViews>
   <sheets>
-    <sheet name="Template Version 2" sheetId="5" r:id="rId1"/>
-    <sheet name="Template Version 1" sheetId="1" state="hidden" r:id="rId2"/>
+    <sheet name="Change Log" sheetId="6" r:id="rId1"/>
+    <sheet name="Template Version 5" sheetId="5" r:id="rId2"/>
+    <sheet name="Template Version 1" sheetId="1" state="hidden" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="114">
   <si>
     <t>Day</t>
   </si>
@@ -348,9 +349,6 @@
     <t>CM 2 Due On</t>
   </si>
   <si>
-    <t>00/00/00</t>
-  </si>
-  <si>
     <t>Available</t>
   </si>
   <si>
@@ -360,18 +358,43 @@
     <t>Remaining AFTER Attack</t>
   </si>
   <si>
-    <t>1/0/1900</t>
+    <t>Quick Note: https://buymeacoffee.com/theultimatejourney</t>
+  </si>
+  <si>
+    <t>00/00/0000</t>
+  </si>
+  <si>
+    <t>Days Left:</t>
+  </si>
+  <si>
+    <t>Latest Due By Date</t>
+  </si>
+  <si>
+    <t>Change Requested By</t>
+  </si>
+  <si>
+    <t>Assigned To</t>
+  </si>
+  <si>
+    <t>Request</t>
+  </si>
+  <si>
+    <t>BSA Note</t>
+  </si>
+  <si>
+    <t>Completion Date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     <numFmt numFmtId="165" formatCode="mmm\-yyyy"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,6 +440,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF92D050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -496,7 +527,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -582,12 +613,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -805,21 +851,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -830,8 +861,86 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1147,12 +1256,46 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E79790A0-8B41-F94C-92A1-BAEDBA4D0CB1}">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="116" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="116" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" s="116" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="116" t="s">
+        <v>111</v>
+      </c>
+      <c r="E1" s="116" t="s">
+        <v>112</v>
+      </c>
+      <c r="F1" s="116" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE1543BC-89E0-46D1-A050-F10A0CF8D26C}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:W51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="43.5" customWidth="1"/>
+    <col min="1" max="1" width="47" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
@@ -1177,7 +1320,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="92"/>
+      <c r="A1" s="115"/>
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -1204,27 +1347,29 @@
       </c>
     </row>
     <row r="2" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="92"/>
+      <c r="A2" s="115"/>
       <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
       <c r="D2" s="5">
         <v>0</v>
       </c>
-      <c r="E2" s="9">
-        <v>0</v>
-      </c>
-      <c r="F2" s="7">
-        <v>0</v>
-      </c>
-      <c r="G2" s="8">
+      <c r="E2" s="89">
+        <v>0</v>
+      </c>
+      <c r="F2" s="90">
+        <v>0</v>
+      </c>
+      <c r="G2" s="92">
         <f>D3</f>
         <v>0</v>
       </c>
-      <c r="H2" s="6">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6">
-        <f>E2+G2</f>
+      <c r="H2" s="91">
+        <v>0</v>
+      </c>
+      <c r="I2" s="91">
+        <f>B13+B14</f>
         <v>0</v>
       </c>
       <c r="J2" s="9"/>
@@ -1236,27 +1381,27 @@
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:17" ht="33" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="92"/>
+      <c r="A3" s="115"/>
       <c r="B3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="93">
         <f>IF(J23&gt;L23,D3,D3-(L23-J23)+G17)</f>
         <v>0</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="95">
         <v>0</v>
       </c>
       <c r="E3" s="3"/>
-      <c r="F3" s="6">
+      <c r="F3" s="91">
         <f>-F2+500</f>
         <v>500</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="91">
         <f>E2</f>
         <v>0</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="91">
         <f>F2+C9</f>
         <v>0</v>
       </c>
@@ -1265,37 +1410,37 @@
       </c>
       <c r="K3" s="14"/>
       <c r="Q3" s="2" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="92"/>
+      <c r="A4" s="115"/>
       <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="91">
         <f>D25+D26</f>
         <v>0</v>
       </c>
-      <c r="D4" s="22">
-        <v>0</v>
-      </c>
-      <c r="E4" s="27" t="s">
+      <c r="D4" s="96" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="97" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="114">
         <f>F3+F2</f>
         <v>500</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="114">
         <f>G2+G3</f>
         <v>0</v>
       </c>
-      <c r="I4" s="17">
+      <c r="I4" s="112">
         <f>SUM(I2:I3)</f>
         <v>0</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="111">
         <f>B12+I4+G17</f>
         <v>0</v>
       </c>
@@ -1314,24 +1459,23 @@
       <c r="P4" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="Q4" s="14">
-        <f>H$13</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="92"/>
+      <c r="Q4" s="29" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="19" x14ac:dyDescent="0.25">
+      <c r="A5" s="115"/>
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="91">
         <f>SUM(D5:E5)-E11</f>
         <v>0</v>
       </c>
-      <c r="D5" s="22">
-        <v>0</v>
-      </c>
-      <c r="E5" s="24">
+      <c r="D5" s="96">
+        <v>0</v>
+      </c>
+      <c r="E5" s="98">
         <v>0</v>
       </c>
       <c r="F5" s="10" t="s">
@@ -1348,17 +1492,20 @@
       <c r="O5" s="10">
         <v>-7500</v>
       </c>
-      <c r="P5" s="26" t="str">
-        <f>IF(J$4&lt;O5, "&lt;", "")</f>
-        <v/>
+      <c r="P5" s="45" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q5" s="88" t="e">
+        <f ca="1">MAX(0,Q4-TODAY())</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="92"/>
+      <c r="A6" s="115"/>
       <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="91">
         <f>D27</f>
         <v>0</v>
       </c>
@@ -1387,11 +1534,11 @@
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="92"/>
+      <c r="A7" s="115"/>
       <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="91">
         <f t="shared" ref="C7:C8" si="3">D28</f>
         <v>0</v>
       </c>
@@ -1421,11 +1568,11 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="92"/>
+      <c r="A8" s="115"/>
       <c r="B8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="91">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1455,11 +1602,11 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="92"/>
+      <c r="A9" s="115"/>
       <c r="B9" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="81">
+      <c r="C9" s="94">
         <f>SUM(D9:E9)</f>
         <v>0</v>
       </c>
@@ -1492,7 +1639,7 @@
       <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="91">
         <f>C3</f>
         <v>0</v>
       </c>
@@ -1518,10 +1665,10 @@
     </row>
     <row r="11" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>105</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C11" s="28" t="str">
         <f>IF(B13&gt;0,"There is a CM Approaching","All Clear")</f>
@@ -1530,12 +1677,12 @@
       <c r="D11" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="89">
         <f>F6+F7+F8+F9</f>
         <v>0</v>
       </c>
-      <c r="H11" s="29">
-        <v>0</v>
+      <c r="H11" s="29" t="s">
+        <v>106</v>
       </c>
       <c r="M11" s="19" t="str">
         <f t="shared" si="0"/>
@@ -1569,7 +1716,7 @@
         <v>31</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>33</v>
@@ -1607,42 +1754,42 @@
       <c r="A13" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="22">
-        <v>0</v>
-      </c>
-      <c r="C13" s="35">
-        <v>0</v>
-      </c>
-      <c r="D13" s="22">
+      <c r="B13" s="96">
+        <v>0</v>
+      </c>
+      <c r="C13" s="99">
+        <v>0</v>
+      </c>
+      <c r="D13" s="96">
         <f>B13-C13</f>
         <v>0</v>
       </c>
-      <c r="E13" s="36">
+      <c r="E13" s="100">
         <f>I13</f>
         <v>0</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="96">
         <f>B13-E13</f>
         <v>0</v>
       </c>
-      <c r="G13" s="37">
-        <f>H13-C2</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="38">
-        <v>0</v>
-      </c>
-      <c r="I13" s="22">
-        <v>0</v>
-      </c>
-      <c r="J13" s="24">
+      <c r="G13" s="37" t="str">
+        <f>IFERROR(IF(OR(H13=0,C2=0),"",H13-C2),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="I13" s="96">
+        <v>0</v>
+      </c>
+      <c r="J13" s="98">
         <f>L13</f>
         <v>0</v>
       </c>
       <c r="K13" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L13" s="22">
+      <c r="L13" s="96">
         <f>C13</f>
         <v>0</v>
       </c>
@@ -1664,42 +1811,42 @@
       <c r="A14" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="22">
-        <v>0</v>
-      </c>
-      <c r="C14" s="35">
-        <v>0</v>
-      </c>
-      <c r="D14" s="22">
+      <c r="B14" s="96">
+        <v>0</v>
+      </c>
+      <c r="C14" s="99">
+        <v>0</v>
+      </c>
+      <c r="D14" s="96">
         <f>B14-C14</f>
         <v>0</v>
       </c>
-      <c r="E14" s="36">
+      <c r="E14" s="100">
         <f>I14</f>
         <v>0</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="96">
         <f>B14-E14</f>
         <v>0</v>
       </c>
-      <c r="G14" s="37" t="e">
-        <f>H14-C2</f>
-        <v>#VALUE!</v>
+      <c r="G14" s="37" t="str">
+        <f>IFERROR(IF(OR(H14=0,C2=0),"",H14-C2),"")</f>
+        <v/>
       </c>
       <c r="H14" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="I14" s="22">
-        <v>0</v>
-      </c>
-      <c r="J14" s="24">
+      <c r="I14" s="96">
+        <v>0</v>
+      </c>
+      <c r="J14" s="98">
         <f>L14</f>
         <v>0</v>
       </c>
       <c r="K14" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L14" s="22">
+      <c r="L14" s="96">
         <f>C14</f>
         <v>0</v>
       </c>
@@ -1721,23 +1868,23 @@
       <c r="A15" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="58">
+      <c r="B15" s="93">
         <f>SUM(B13:B14)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="35">
+      <c r="C15" s="99">
         <f>SUM(C13:C14)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="96">
         <f>SUM(D13:D14)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="100">
         <f>SUM(E13:E14)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="40">
+      <c r="F15" s="101">
         <f>SUM(F13:F14)</f>
         <v>0</v>
       </c>
@@ -1745,18 +1892,18 @@
       <c r="H15" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="I15" s="41">
+      <c r="I15" s="102">
         <f>SUM(I13:I14)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="24">
+      <c r="J15" s="98">
         <f>SUM(J13:J14)</f>
         <v>0</v>
       </c>
       <c r="K15" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L15" s="22">
+      <c r="L15" s="96">
         <f>SUM(L13:L14)</f>
         <v>0</v>
       </c>
@@ -1800,7 +1947,7 @@
       <c r="A17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="46">
+      <c r="B17" s="103">
         <v>0</v>
       </c>
       <c r="C17" s="10" t="s">
@@ -1832,14 +1979,14 @@
       <c r="A18">
         <v>1</v>
       </c>
-      <c r="B18" s="46">
+      <c r="B18" s="103">
         <v>0</v>
       </c>
       <c r="C18" s="15" t="str">
         <f>IF(B28&gt;B17,"Increase","Decrease")</f>
         <v>Decrease</v>
       </c>
-      <c r="D18" s="51">
+      <c r="D18" s="105">
         <f>B28-B17</f>
         <v>0</v>
       </c>
@@ -1867,16 +2014,16 @@
       <c r="A19">
         <v>2</v>
       </c>
-      <c r="B19" s="46">
+      <c r="B19" s="103">
         <v>0</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="52">
+      <c r="F19" s="52" t="str">
         <f>H11</f>
-        <v>0</v>
+        <v>00/00/0000</v>
       </c>
       <c r="G19" s="10"/>
       <c r="H19" s="15" t="s">
@@ -1888,9 +2035,9 @@
       <c r="K19" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="L19" s="53">
+      <c r="L19" s="53" t="str">
         <f>H13</f>
-        <v>0</v>
+        <v>00/00/0000</v>
       </c>
       <c r="M19" s="19" t="str">
         <f t="shared" si="0"/>
@@ -1910,7 +2057,7 @@
       <c r="A20">
         <v>3</v>
       </c>
-      <c r="B20" s="46">
+      <c r="B20" s="96">
         <v>0</v>
       </c>
       <c r="D20" s="10"/>
@@ -1927,15 +2074,15 @@
       <c r="I20" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="J20" s="57">
-        <f>I15</f>
+      <c r="J20" s="104">
+        <f>J15</f>
         <v>0</v>
       </c>
       <c r="K20" s="54" t="str">
         <f>IF(J20 &gt;=L20, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L20" s="58">
+      <c r="L20" s="93">
         <f>L15</f>
         <v>0</v>
       </c>
@@ -1957,26 +2104,26 @@
       <c r="A21">
         <v>4</v>
       </c>
-      <c r="B21" s="46">
+      <c r="B21" s="96">
         <v>0</v>
       </c>
       <c r="D21" s="10"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="59">
+      <c r="F21" s="59" t="str">
         <f>H13</f>
-        <v>0</v>
-      </c>
-      <c r="G21" s="82">
-        <f>F21-E23</f>
-        <v>0</v>
-      </c>
-      <c r="H21" s="88" t="s">
+        <v>00/00/0000</v>
+      </c>
+      <c r="G21" s="82" t="str">
+        <f>IFERROR(IF(OR(F21=0,E23=0),"",F21-E23),"")</f>
+        <v/>
+      </c>
+      <c r="H21" s="83" t="s">
         <v>98</v>
       </c>
       <c r="I21" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="J21" s="58">
+      <c r="J21" s="93">
         <f>D25</f>
         <v>0</v>
       </c>
@@ -1984,7 +2131,7 @@
         <f>IF(J21 =L21, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L21" s="58">
+      <c r="L21" s="93">
         <f>D25</f>
         <v>0</v>
       </c>
@@ -2006,7 +2153,8 @@
       <c r="A22">
         <v>5</v>
       </c>
-      <c r="B22" s="46">
+      <c r="B22" s="96">
+        <f t="shared" ref="B22" si="4">SUM(B17:B21)</f>
         <v>0</v>
       </c>
       <c r="D22" s="10"/>
@@ -2023,7 +2171,7 @@
       <c r="I22" s="56" t="s">
         <v>60</v>
       </c>
-      <c r="J22" s="57">
+      <c r="J22" s="104">
         <f>D26</f>
         <v>0</v>
       </c>
@@ -2031,7 +2179,7 @@
         <f>IF(J22 =L22, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L22" s="58">
+      <c r="L22" s="93">
         <f>D26</f>
         <v>0</v>
       </c>
@@ -2053,7 +2201,7 @@
       <c r="A23">
         <v>6</v>
       </c>
-      <c r="B23" s="46">
+      <c r="B23" s="103">
         <v>0</v>
       </c>
       <c r="D23" s="10"/>
@@ -2061,20 +2209,21 @@
         <f>C2</f>
         <v>0</v>
       </c>
-      <c r="F23" s="61" t="s">
+      <c r="F23" s="61" t="str">
+        <f>H14</f>
+        <v>00/00/0000</v>
+      </c>
+      <c r="G23" s="82" t="str">
+        <f>IFERROR(IF(OR(F23=0,E23=0),"",F23-E23),"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="83" t="s">
+        <v>97</v>
+      </c>
+      <c r="I23" s="58" t="s">
         <v>102</v>
       </c>
-      <c r="G23" s="82" t="e">
-        <f>IMSUB(F23,E23)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="H23" s="88" t="s">
-        <v>97</v>
-      </c>
-      <c r="I23" s="58" t="s">
-        <v>103</v>
-      </c>
-      <c r="J23" s="18">
+      <c r="J23" s="111">
         <f>SUM(J20:J22)</f>
         <v>0</v>
       </c>
@@ -2082,7 +2231,7 @@
         <f>IF(J23 =L23, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L23" s="58">
+      <c r="L23" s="93">
         <f>SUM(L20:L22)</f>
         <v>0</v>
       </c>
@@ -2104,7 +2253,7 @@
       <c r="A24">
         <v>7</v>
       </c>
-      <c r="B24" s="46">
+      <c r="B24" s="103">
         <v>0</v>
       </c>
       <c r="C24" s="15" t="s">
@@ -2114,12 +2263,12 @@
       <c r="E24" s="62" t="s">
         <v>99</v>
       </c>
-      <c r="G24" s="89"/>
-      <c r="H24" s="89"/>
-      <c r="I24" s="90"/>
-      <c r="J24" s="91"/>
+      <c r="G24" s="84"/>
+      <c r="H24" s="84"/>
+      <c r="I24" s="85"/>
+      <c r="J24" s="86"/>
       <c r="K24" s="72"/>
-      <c r="L24" s="89"/>
+      <c r="L24" s="84"/>
       <c r="M24" s="19" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2138,24 +2287,24 @@
       <c r="A25">
         <v>8</v>
       </c>
-      <c r="B25" s="46">
+      <c r="B25" s="103">
         <v>0</v>
       </c>
       <c r="C25" s="2" t="str">
         <f>I21</f>
         <v>Mortgage</v>
       </c>
-      <c r="D25" s="62">
-        <v>0</v>
-      </c>
-      <c r="E25" s="4">
+      <c r="D25" s="103">
+        <v>0</v>
+      </c>
+      <c r="E25" s="87">
         <f>C$2</f>
         <v>0</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="83">
+      <c r="H25" s="106">
         <f>F2</f>
         <v>0</v>
       </c>
@@ -2189,33 +2338,33 @@
       <c r="A26">
         <v>9</v>
       </c>
-      <c r="B26" s="46">
+      <c r="B26" s="96">
         <v>0</v>
       </c>
       <c r="C26" s="2" t="str">
         <f>I22</f>
         <v>HOA</v>
       </c>
-      <c r="D26" s="62">
-        <v>0</v>
-      </c>
-      <c r="E26" s="4">
-        <f t="shared" ref="E26:E29" si="4">C$2</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="84">
+      <c r="D26" s="103">
+        <v>0</v>
+      </c>
+      <c r="E26" s="87">
+        <f t="shared" ref="E26:E29" si="5">C$2</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="107">
         <f>G2</f>
         <v>0</v>
       </c>
-      <c r="I26" s="66">
+      <c r="I26" s="98">
         <f>G17+C3+F2-I15-M50+E11</f>
         <v>0</v>
       </c>
-      <c r="J26" s="66">
+      <c r="J26" s="98">
         <f>G17+C3+C8+F2-M50</f>
         <v>0</v>
       </c>
-      <c r="K26" s="67">
+      <c r="K26" s="113">
         <v>5000</v>
       </c>
       <c r="L26" s="68" t="str">
@@ -2240,24 +2389,24 @@
       <c r="A27">
         <v>10</v>
       </c>
-      <c r="B27" s="46">
+      <c r="B27" s="96">
         <v>0</v>
       </c>
       <c r="C27" s="2" t="str">
         <f>B6</f>
         <v>Vacation Savings</v>
       </c>
-      <c r="D27" s="62">
-        <v>0</v>
-      </c>
-      <c r="E27" s="4">
-        <f t="shared" si="4"/>
+      <c r="D27" s="103">
+        <v>0</v>
+      </c>
+      <c r="E27" s="87">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G27" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="H27" s="85">
+      <c r="H27" s="108">
         <f>SUM(H25:H26)</f>
         <v>0</v>
       </c>
@@ -2283,24 +2432,25 @@
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="46">
+      <c r="B28" s="96">
+        <f t="shared" ref="B28" si="6">SUM(B23:B27)</f>
         <v>0</v>
       </c>
       <c r="C28" s="2" t="str">
         <f>B7</f>
         <v>Emergency Savings</v>
       </c>
-      <c r="D28" s="22">
-        <v>0</v>
-      </c>
-      <c r="E28" s="4">
-        <f t="shared" si="4"/>
+      <c r="D28" s="96">
+        <v>0</v>
+      </c>
+      <c r="E28" s="87">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="H28" s="86">
+      <c r="H28" s="109">
         <f>H27-D30</f>
         <v>0</v>
       </c>
@@ -2329,17 +2479,17 @@
         <f>B8</f>
         <v>Boost Savings</v>
       </c>
-      <c r="D29" s="22">
-        <v>0</v>
-      </c>
-      <c r="E29" s="4">
-        <f t="shared" si="4"/>
+      <c r="D29" s="96">
+        <v>0</v>
+      </c>
+      <c r="E29" s="87">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G29" t="s">
         <v>71</v>
       </c>
-      <c r="H29" s="87">
+      <c r="H29" s="110">
         <f>H27+G17</f>
         <v>0</v>
       </c>
@@ -2362,10 +2512,11 @@
       <c r="Q29" s="30"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="B30" s="117"/>
       <c r="C30" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="22">
+      <c r="D30" s="96">
         <f>SUM(D25:D29)</f>
         <v>0</v>
       </c>
@@ -2389,6 +2540,7 @@
       <c r="Q30" s="30"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="B31" s="22"/>
       <c r="C31" s="2"/>
       <c r="D31" s="10"/>
       <c r="H31" s="10"/>
@@ -2403,6 +2555,7 @@
       <c r="Q31" s="10"/>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="B32" s="6"/>
       <c r="H32" s="10"/>
       <c r="I32" s="10"/>
       <c r="J32" s="13"/>
@@ -2415,31 +2568,17 @@
       <c r="Q32" s="10"/>
       <c r="W32" s="10"/>
     </row>
-    <row r="33" spans="1:20" ht="32" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:20" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="E33" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F33" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="G33" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="H33" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="I33" s="27" t="s">
-        <v>79</v>
-      </c>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27"/>
       <c r="J33" s="15"/>
       <c r="K33" s="15" t="s">
         <v>80</v>
@@ -2479,20 +2618,20 @@
       <c r="L34" s="72"/>
       <c r="M34" s="69"/>
       <c r="N34" s="74">
-        <f>I26</f>
-        <v>0</v>
-      </c>
-      <c r="O34" s="37" t="e">
-        <f>N34/Q50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P34" s="37" t="e">
-        <f>O34/Q50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q34" s="37" t="e">
-        <f>P34/Q50</f>
-        <v>#DIV/0!</v>
+        <f>IFERROR(I26,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O34" s="37">
+        <f>IFERROR(N34/Q50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P34" s="37">
+        <f>IFERROR(O34/Q50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q34" s="37">
+        <f>IFERROR(P34/Q50,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.2">
@@ -2513,25 +2652,25 @@
       <c r="J35" s="76"/>
       <c r="K35" s="76"/>
       <c r="L35" s="76"/>
-      <c r="M35" s="57">
-        <f t="shared" ref="M35" si="5">SUM(C35:I35)</f>
+      <c r="M35" s="104">
+        <f t="shared" ref="M35" si="7">SUM(C35:I35)</f>
         <v>0</v>
       </c>
       <c r="N35" s="77">
-        <f>N34-M35</f>
-        <v>0</v>
-      </c>
-      <c r="O35" s="77" t="e">
-        <f>O34-M35/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P35" s="77" t="e">
-        <f>P34-M35/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q35" s="77" t="e">
-        <f>Q34-M35/Q$50</f>
-        <v>#DIV/0!</v>
+        <f>IFERROR(N34-M35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O35" s="77">
+        <f t="shared" ref="O35:O48" si="8">IFERROR(O34-M35/Q$50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P35" s="77">
+        <f t="shared" ref="P35:P48" si="9">IFERROR(P34-M35/Q$50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q35" s="77">
+        <f t="shared" ref="Q35:Q48" si="10">IFERROR(Q34-M35/Q$50,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.2">
@@ -2552,25 +2691,25 @@
       <c r="J36" s="76"/>
       <c r="K36" s="76"/>
       <c r="L36" s="76"/>
-      <c r="M36" s="57">
+      <c r="M36" s="104">
         <f>SUM(C36:L36)</f>
         <v>0</v>
       </c>
-      <c r="N36" s="77" t="e">
-        <f>N35-M36/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O36" s="77" t="e">
-        <f t="shared" ref="O36:O48" si="6">O35-M36/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P36" s="77" t="e">
-        <f t="shared" ref="P36:P48" si="7">P35-M36/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q36" s="77" t="e">
-        <f t="shared" ref="Q36:Q48" si="8">Q35-M36/Q$50</f>
-        <v>#DIV/0!</v>
+      <c r="N36" s="77">
+        <f t="shared" ref="N36:N48" si="11">IFERROR(N35-M36/Q$50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O36" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P36" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q36" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.2">
@@ -2591,25 +2730,25 @@
       <c r="J37" s="76"/>
       <c r="K37" s="76"/>
       <c r="L37" s="76"/>
-      <c r="M37" s="57">
+      <c r="M37" s="104">
         <f>SUM(C37:L37)</f>
         <v>0</v>
       </c>
-      <c r="N37" s="77" t="e">
-        <f t="shared" ref="N37:N48" si="9">N36-M37/Q$50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O37" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P37" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q37" s="77" t="e">
+      <c r="N37" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O37" s="77">
         <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="P37" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q37" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.2">
@@ -2630,25 +2769,25 @@
       <c r="J38" s="76"/>
       <c r="K38" s="76"/>
       <c r="L38" s="76"/>
-      <c r="M38" s="57">
-        <f t="shared" ref="M38:M48" si="10">SUM(C38:L38)</f>
-        <v>0</v>
-      </c>
-      <c r="N38" s="77" t="e">
+      <c r="M38" s="104">
+        <f t="shared" ref="M38:M48" si="12">SUM(C38:L38)</f>
+        <v>0</v>
+      </c>
+      <c r="N38" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O38" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P38" s="77">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O38" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P38" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q38" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="Q38" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.2">
@@ -2669,25 +2808,25 @@
       <c r="J39" s="76"/>
       <c r="K39" s="76"/>
       <c r="L39" s="76"/>
-      <c r="M39" s="57">
+      <c r="M39" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N39" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O39" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P39" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q39" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N39" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O39" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P39" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q39" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="40" spans="1:20" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2708,25 +2847,25 @@
       <c r="J40" s="76"/>
       <c r="K40" s="76"/>
       <c r="L40" s="76"/>
-      <c r="M40" s="57">
+      <c r="M40" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N40" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O40" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P40" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q40" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N40" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O40" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P40" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q40" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="41" spans="1:20" ht="12" customHeight="1" x14ac:dyDescent="0.2">
@@ -2747,25 +2886,25 @@
       <c r="J41" s="76"/>
       <c r="K41" s="76"/>
       <c r="L41" s="76"/>
-      <c r="M41" s="57">
+      <c r="M41" s="104">
         <f>SUM(C41:L41)</f>
         <v>0</v>
       </c>
-      <c r="N41" s="77" t="e">
+      <c r="N41" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O41" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P41" s="77">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O41" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P41" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q41" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="Q41" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.2">
@@ -2786,25 +2925,25 @@
       <c r="J42" s="76"/>
       <c r="K42" s="76"/>
       <c r="L42" s="76"/>
-      <c r="M42" s="57">
+      <c r="M42" s="104">
         <f>SUM(C42:L42)</f>
         <v>0</v>
       </c>
-      <c r="N42" s="77" t="e">
+      <c r="N42" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O42" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P42" s="77">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O42" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P42" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q42" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="Q42" s="77">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.2">
@@ -2825,25 +2964,25 @@
       <c r="J43" s="76"/>
       <c r="K43" s="76"/>
       <c r="L43" s="76"/>
-      <c r="M43" s="57">
+      <c r="M43" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N43" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O43" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P43" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q43" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N43" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O43" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P43" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q43" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.2">
@@ -2864,25 +3003,25 @@
       <c r="J44" s="76"/>
       <c r="K44" s="76"/>
       <c r="L44" s="76"/>
-      <c r="M44" s="57">
+      <c r="M44" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N44" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O44" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P44" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q44" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N44" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O44" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P44" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q44" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.2">
@@ -2903,25 +3042,25 @@
       <c r="J45" s="76"/>
       <c r="K45" s="76"/>
       <c r="L45" s="76"/>
-      <c r="M45" s="57">
+      <c r="M45" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N45" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O45" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P45" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q45" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N45" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O45" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P45" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q45" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.2">
@@ -2942,25 +3081,25 @@
       <c r="J46" s="76"/>
       <c r="K46" s="76"/>
       <c r="L46" s="76"/>
-      <c r="M46" s="57">
+      <c r="M46" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N46" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O46" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P46" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q46" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N46" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O46" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P46" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q46" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.2">
@@ -2981,25 +3120,25 @@
       <c r="J47" s="76"/>
       <c r="K47" s="76"/>
       <c r="L47" s="76"/>
-      <c r="M47" s="57">
+      <c r="M47" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N47" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O47" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P47" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q47" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N47" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O47" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P47" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q47" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.2">
@@ -3020,25 +3159,25 @@
       <c r="J48" s="78"/>
       <c r="K48" s="78"/>
       <c r="L48" s="78"/>
-      <c r="M48" s="57">
+      <c r="M48" s="104">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N48" s="77">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O48" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P48" s="77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="Q48" s="77">
         <f t="shared" si="10"/>
         <v>0</v>
-      </c>
-      <c r="N48" s="77" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O48" s="77" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P48" s="77" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q48" s="77" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="49" spans="2:17" x14ac:dyDescent="0.2">
@@ -3071,61 +3210,61 @@
       <c r="B50" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C50" s="62">
+      <c r="C50" s="103">
         <f>SUM(C35:C48)</f>
         <v>0</v>
       </c>
-      <c r="D50" s="62">
+      <c r="D50" s="103">
         <f>SUM(D35:D48)</f>
         <v>0</v>
       </c>
-      <c r="E50" s="62">
-        <f t="shared" ref="E50:L50" si="11">SUM(E36:E48)</f>
-        <v>0</v>
-      </c>
-      <c r="F50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="G50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="H50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="K50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="L50" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="M50" s="62">
+      <c r="E50" s="103">
+        <f t="shared" ref="E50:L50" si="13">SUM(E36:E48)</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="H50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="I50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="K50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="L50" s="103">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="M50" s="103">
         <f>SUM(M35:M48)</f>
         <v>0</v>
       </c>
-      <c r="N50" s="80" t="e">
-        <f>I26/H27</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O50" s="37" t="e">
-        <f>(N34-M50)/Q50</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P50" s="80" t="e">
-        <f>100% -N50</f>
-        <v>#DIV/0!</v>
+      <c r="N50" s="80">
+        <f>IFERROR(I26/H27,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O50" s="37">
+        <f>IFERROR((N34-M50)/Q50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P50" s="80">
+        <f>IFERROR(100% -N50,0)</f>
+        <v>1</v>
       </c>
       <c r="Q50" s="15">
         <f>G19</f>
@@ -3139,11 +3278,200 @@
   <mergeCells count="1">
     <mergeCell ref="A1:A9"/>
   </mergeCells>
+  <dataValidations count="47">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{3170D0ED-69B8-2147-B2E8-C845548A1AEB}">
+      <formula1>"Monday,Tuesday,Wednesday,Thursday,Friday,Saturday,Sunday"</formula1>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="Date Entry" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="C2" xr:uid="{1A0AC821-D2F1-CC47-BCD2-867E6217E64D}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Time" error="Please enter a valid time format (e.g., 11:22 AM, 14:30)" promptTitle="Time Entry" prompt="Please enter a valid time (e.g., 11:22 AM, 14:30, 8:08:00 AM)" sqref="D2" xr:uid="{725F1B26-DEA2-2544-B362-19E809BAA3B2}">
+      <formula1>0</formula1>
+      <formula2>0.999988425925926</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount (numbers only, e.g., 100.00)" promptTitle="Saved Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="E2" xr:uid="{554C6FD8-DF46-C24A-B6DA-75188B87833F}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount (numbers only)." promptTitle="Fuel Amount" prompt="Please enter a dollar amount for fuel (e.g., 50.00, 125.75)" sqref="F2" xr:uid="{2945CFF3-B39B-6B4D-A81C-A094F8872C7D}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount (number between 0 and 999,999,999.99)" promptTitle="Bank Saved Amount" prompt="Please enter a dollar amount for bank savings (e.g., 100.00, 250.50)" sqref="H2" xr:uid="{DEBEAC84-DA60-D443-A7D6-80BC8F319DBE}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="This cell contains a formula. Please edit E2 or G2 instead." promptTitle="Total Credit Card" prompt="This cell calculates the total credit card amount (Saved + Bank)" sqref="I2" xr:uid="{827C1756-1326-E340-9238-09B695E4E03F}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format (e.g., 5/15/2026)" promptTitle="Estimated Pay Drop Date" prompt="Please enter a valid date (e.g., 5/15/2026)" sqref="H11" xr:uid="{C44A92CA-E0FA-D342-848B-7ED51D8B7AC0}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format (e.g., 5/15/2026)" promptTitle="CM1 Final Due Date" prompt="Please enter a valid date (e.g., 5/15/2026)" sqref="H13 Q4" xr:uid="{9EAB60B5-5BA8-BE43-A9E2-5E5AD8961415}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format (e.g., 5/15/2026)" promptTitle="CM2 Final Due Date" prompt="Please enter a valid date (e.g., 5/15/2026)" sqref="H14" xr:uid="{0B4F1CA8-E9A3-5D46-B4E6-DCA330C9E728}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="As-Of Date (Mortgage)" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E25" xr:uid="{7F9B15EE-805C-624E-91F2-9EE5908FEB8A}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="As-Of Date (Boost Savings)" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E29" xr:uid="{9F0D187E-AECB-354E-B9D0-BBAA1D17C71F}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="Predicted Pay Drop Date" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="F19" xr:uid="{445E3649-2EF6-1244-A502-5986D5BA3DC7}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="CM 1 Due On" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="F21" xr:uid="{F6374D57-9877-D84B-A7A4-1D340524520C}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="CM 2 Due On" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="F23" xr:uid="{20D8721C-CF38-E64D-8EFB-354FA49959E5}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Bank Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="G2" xr:uid="{092CE826-655A-6846-8640-3ECBD514D949}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="HOA As-Of Date" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E26" xr:uid="{D88F751C-C1C5-1447-B3FC-0DDF32987D38}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="Vacation Savings As-Of Date" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E27" xr:uid="{2B6E4F52-F607-7849-AEE9-FBE9DE40A560}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Date" error="Please enter a valid date format." promptTitle="Emergency Savings As-Of Date" prompt="Please enter a valid date (e.g., 5/4/2026)" sqref="E28" xr:uid="{4F21D987-6066-9943-B4CE-1CE92B09D0EE}">
+      <formula1>1</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Savings Balance" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="C3:C10" xr:uid="{04DC61CC-20BC-7C47-91BB-CF0E0D2EFBA0}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Power Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D3:D5" xr:uid="{E33DAC1B-DC8C-ED4F-A043-40499074E2DF}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Water Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="E4:E5" xr:uid="{6385CA2A-90F8-BF4F-8726-40FB3E8083C6}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Debt Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="B13:B15" xr:uid="{351E97BA-1885-6540-90E2-0E2556D5428F}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Minimum Payment" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="C13:C15" xr:uid="{771F17F6-5CF3-764E-B272-86B3732C43A6}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Left 2 Go" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D13:D15" xr:uid="{AE461F65-120C-C345-8459-89C9BB09BD41}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Next Attack Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="E13:E15" xr:uid="{0069F0C6-E4A6-D14E-AFBF-52C7887ACD3B}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Remaining After Attack" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="F13:F15" xr:uid="{E60786F5-4666-3644-817A-044B60A0FD44}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Payment Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="I13:I15" xr:uid="{6BAC151E-A408-FC45-827B-DA5F226CA5FE}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Last Statement Balance" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J13:J15" xr:uid="{7B5C52C0-D156-EE4A-B1C3-2B3D6CF86CAE}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Next Minimum" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="L13:L15" xr:uid="{286008C8-7A35-FE44-875D-137AB7724D6D}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Tank Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D25:D29 B17:B21 B23:B27" xr:uid="{DCEE984F-F387-8F43-B4D2-7C222E9FA32E}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Monthly Minimum" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J20:J22" xr:uid="{32B0A9CD-D726-F24B-90D9-1712FC70AB38}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="2 Week Spending" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="M35:M48" xr:uid="{F6775EA3-3841-964B-A2C9-51770973A55B}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Holding Tank" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="E11" xr:uid="{E15B848F-7BE5-AD4D-8EA3-DF0181E63A81}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Decrease Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D18" xr:uid="{503BA0B3-FC97-E342-B416-C46429D9BB19}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Total Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="H25:H29" xr:uid="{4C020DF3-0044-6B4E-B44E-AA614A3D44BD}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Tank Total" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D30 B22 B28" xr:uid="{EB99C4F6-A363-7C40-A9E9-F2C68CD7797D}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="CM Total After Full Attack" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J4" xr:uid="{0A6AAE44-CEA8-144B-AB2F-07206831F561}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="I3:I4 G3:G4" xr:uid="{3434CA11-B4B5-F842-9DEE-B9AE2C83E338}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Current POR" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="I26" xr:uid="{79DBCC11-2E7B-524E-ADB7-9AF1D52645FD}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="All In POR" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J26" xr:uid="{CF78B612-016B-DE4B-BF60-EDF66C5A6429}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Target All-In POR (ROI)" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="K26" xr:uid="{5EDB90BD-F221-AA43-9557-DB7F094BD568}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Status Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="L20:L22" xr:uid="{BA49962A-ED1A-484B-90D9-11DC115BAE55}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Available Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="J23" xr:uid="{E948AC32-8BDA-A247-9194-E7061DA8AB0E}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Monthly Minimum Status" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="L23" xr:uid="{156268F1-6A8C-7041-8A11-92E156C7B41F}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Total" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="C50:M50" xr:uid="{9DFD7696-0A1F-9044-B603-6D89D6ED2136}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Use Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="F3:F4" xr:uid="{416CBC7D-C44C-DD46-BE90-9D72426DF971}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8812D7F7-4E2E-4C59-8640-33FA123A4EE8}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:W51"/>

</xml_diff>

<commit_message>
chore(dash-od-1): replace public dashboard workbook with Dashboardv5—DepartureReady [PAL-105]
- Replaces dashboard-v2.xlsx with the Option C aligned workbook
- New file: Dashboardv5—DepartureReady.xlsx (SHA256: 38b1f562...)
- Old file: SHA256 607aec02... archived locally as dashboard-v2.xlsx.archive-20260615
- Sheet naming now aligns with Option C (departure-ready) convention
- BEEHIIV_GIFT_LINK_URL and public route unchanged — same filename

QA Wolf: verify https://thispagedoesnotexist12345.us/dashboard-v2.xlsx
downloads the new workbook post-deployment.
</commit_message>
<xml_diff>
--- a/client/public/dashboard-v2.xlsx
+++ b/client/public/dashboard-v2.xlsx
@@ -5,17 +5,16 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/home/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/home/Documents/TUJ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9788E4-BA60-CC45-B4AE-80E4653188B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F268080-EC5E-CC4E-9D1E-0A6857091287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18160" activeTab="1" xr2:uid="{3A949835-928B-43F0-8F59-3C1F84CFAB50}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18160" xr2:uid="{3A949835-928B-43F0-8F59-3C1F84CFAB50}"/>
   </bookViews>
   <sheets>
-    <sheet name="Change Log" sheetId="6" r:id="rId1"/>
-    <sheet name="Template Version 5" sheetId="5" r:id="rId2"/>
-    <sheet name="Template Version 1" sheetId="1" state="hidden" r:id="rId3"/>
+    <sheet name="Template Version 5" sheetId="5" r:id="rId1"/>
+    <sheet name="Template Version 1" sheetId="1" state="hidden" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="109">
   <si>
     <t>Day</t>
   </si>
@@ -368,21 +367,6 @@
   </si>
   <si>
     <t>Latest Due By Date</t>
-  </si>
-  <si>
-    <t>Change Requested By</t>
-  </si>
-  <si>
-    <t>Assigned To</t>
-  </si>
-  <si>
-    <t>Request</t>
-  </si>
-  <si>
-    <t>BSA Note</t>
-  </si>
-  <si>
-    <t>Completion Date</t>
   </si>
 </sst>
 </file>
@@ -527,7 +511,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -613,21 +597,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -861,6 +830,9 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -935,12 +907,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1256,40 +1227,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E79790A0-8B41-F94C-92A1-BAEDBA4D0CB1}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="116" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="116" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" s="116" t="s">
-        <v>110</v>
-      </c>
-      <c r="D1" s="116" t="s">
-        <v>111</v>
-      </c>
-      <c r="E1" s="116" t="s">
-        <v>112</v>
-      </c>
-      <c r="F1" s="116" t="s">
-        <v>113</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE1543BC-89E0-46D1-A050-F10A0CF8D26C}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:W51"/>
@@ -1320,7 +1257,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="115"/>
+      <c r="A1" s="117"/>
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -1347,7 +1284,7 @@
       </c>
     </row>
     <row r="2" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="115"/>
+      <c r="A2" s="117"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4">
         <v>0</v>
@@ -1355,20 +1292,20 @@
       <c r="D2" s="5">
         <v>0</v>
       </c>
-      <c r="E2" s="89">
-        <v>0</v>
-      </c>
-      <c r="F2" s="90">
-        <v>0</v>
-      </c>
-      <c r="G2" s="92">
+      <c r="E2" s="90">
+        <v>0</v>
+      </c>
+      <c r="F2" s="91">
+        <v>0</v>
+      </c>
+      <c r="G2" s="93">
         <f>D3</f>
         <v>0</v>
       </c>
-      <c r="H2" s="91">
-        <v>0</v>
-      </c>
-      <c r="I2" s="91">
+      <c r="H2" s="92">
+        <v>0</v>
+      </c>
+      <c r="I2" s="92">
         <f>B13+B14</f>
         <v>0</v>
       </c>
@@ -1381,27 +1318,27 @@
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:17" ht="33" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="115"/>
+      <c r="A3" s="117"/>
       <c r="B3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="93">
+      <c r="C3" s="94">
         <f>IF(J23&gt;L23,D3,D3-(L23-J23)+G17)</f>
         <v>0</v>
       </c>
-      <c r="D3" s="95">
+      <c r="D3" s="96">
         <v>0</v>
       </c>
       <c r="E3" s="3"/>
-      <c r="F3" s="91">
+      <c r="F3" s="92">
         <f>-F2+500</f>
         <v>500</v>
       </c>
-      <c r="G3" s="91">
+      <c r="G3" s="92">
         <f>E2</f>
         <v>0</v>
       </c>
-      <c r="I3" s="91">
+      <c r="I3" s="92">
         <f>F2+C9</f>
         <v>0</v>
       </c>
@@ -1414,33 +1351,33 @@
       </c>
     </row>
     <row r="4" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="115"/>
+      <c r="A4" s="117"/>
       <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="91">
+      <c r="C4" s="92">
         <f>D25+D26</f>
         <v>0</v>
       </c>
-      <c r="D4" s="96" t="s">
+      <c r="D4" s="97" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="97" t="s">
+      <c r="E4" s="98" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="114">
+      <c r="F4" s="115">
         <f>F3+F2</f>
         <v>500</v>
       </c>
-      <c r="G4" s="114">
+      <c r="G4" s="115">
         <f>G2+G3</f>
         <v>0</v>
       </c>
-      <c r="I4" s="112">
+      <c r="I4" s="113">
         <f>SUM(I2:I3)</f>
         <v>0</v>
       </c>
-      <c r="J4" s="111">
+      <c r="J4" s="112">
         <f>B12+I4+G17</f>
         <v>0</v>
       </c>
@@ -1464,18 +1401,18 @@
       </c>
     </row>
     <row r="5" spans="1:17" ht="19" x14ac:dyDescent="0.25">
-      <c r="A5" s="115"/>
+      <c r="A5" s="117"/>
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="91">
+      <c r="C5" s="92">
         <f>SUM(D5:E5)-E11</f>
         <v>0</v>
       </c>
-      <c r="D5" s="96">
-        <v>0</v>
-      </c>
-      <c r="E5" s="98">
+      <c r="D5" s="97">
+        <v>0</v>
+      </c>
+      <c r="E5" s="99">
         <v>0</v>
       </c>
       <c r="F5" s="10" t="s">
@@ -1495,17 +1432,17 @@
       <c r="P5" s="45" t="s">
         <v>107</v>
       </c>
-      <c r="Q5" s="88" t="e">
+      <c r="Q5" s="89" t="e">
         <f ca="1">MAX(0,Q4-TODAY())</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="115"/>
+      <c r="A6" s="117"/>
       <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="91">
+      <c r="C6" s="92">
         <f>D27</f>
         <v>0</v>
       </c>
@@ -1534,11 +1471,11 @@
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="115"/>
+      <c r="A7" s="117"/>
       <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="91">
+      <c r="C7" s="92">
         <f t="shared" ref="C7:C8" si="3">D28</f>
         <v>0</v>
       </c>
@@ -1568,11 +1505,11 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="115"/>
+      <c r="A8" s="117"/>
       <c r="B8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="91">
+      <c r="C8" s="92">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1602,11 +1539,11 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="115"/>
+      <c r="A9" s="117"/>
       <c r="B9" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="94">
+      <c r="C9" s="95">
         <f>SUM(D9:E9)</f>
         <v>0</v>
       </c>
@@ -1639,7 +1576,7 @@
       <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="91">
+      <c r="C10" s="92">
         <f>C3</f>
         <v>0</v>
       </c>
@@ -1677,7 +1614,7 @@
       <c r="D11" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="89">
+      <c r="E11" s="90">
         <f>F6+F7+F8+F9</f>
         <v>0</v>
       </c>
@@ -1754,21 +1691,21 @@
       <c r="A13" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="96">
-        <v>0</v>
-      </c>
-      <c r="C13" s="99">
-        <v>0</v>
-      </c>
-      <c r="D13" s="96">
+      <c r="B13" s="97">
+        <v>0</v>
+      </c>
+      <c r="C13" s="100">
+        <v>0</v>
+      </c>
+      <c r="D13" s="97">
         <f>B13-C13</f>
         <v>0</v>
       </c>
-      <c r="E13" s="100">
+      <c r="E13" s="101">
         <f>I13</f>
         <v>0</v>
       </c>
-      <c r="F13" s="96">
+      <c r="F13" s="97">
         <f>B13-E13</f>
         <v>0</v>
       </c>
@@ -1779,17 +1716,17 @@
       <c r="H13" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="I13" s="96">
-        <v>0</v>
-      </c>
-      <c r="J13" s="98">
+      <c r="I13" s="97">
+        <v>0</v>
+      </c>
+      <c r="J13" s="99">
         <f>L13</f>
         <v>0</v>
       </c>
       <c r="K13" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L13" s="96">
+      <c r="L13" s="97">
         <f>C13</f>
         <v>0</v>
       </c>
@@ -1811,21 +1748,21 @@
       <c r="A14" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="96">
-        <v>0</v>
-      </c>
-      <c r="C14" s="99">
-        <v>0</v>
-      </c>
-      <c r="D14" s="96">
+      <c r="B14" s="97">
+        <v>0</v>
+      </c>
+      <c r="C14" s="100">
+        <v>0</v>
+      </c>
+      <c r="D14" s="97">
         <f>B14-C14</f>
         <v>0</v>
       </c>
-      <c r="E14" s="100">
+      <c r="E14" s="101">
         <f>I14</f>
         <v>0</v>
       </c>
-      <c r="F14" s="96">
+      <c r="F14" s="97">
         <f>B14-E14</f>
         <v>0</v>
       </c>
@@ -1836,17 +1773,17 @@
       <c r="H14" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="I14" s="96">
-        <v>0</v>
-      </c>
-      <c r="J14" s="98">
+      <c r="I14" s="97">
+        <v>0</v>
+      </c>
+      <c r="J14" s="99">
         <f>L14</f>
         <v>0</v>
       </c>
       <c r="K14" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L14" s="96">
+      <c r="L14" s="97">
         <f>C14</f>
         <v>0</v>
       </c>
@@ -1868,23 +1805,23 @@
       <c r="A15" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="93">
+      <c r="B15" s="94">
         <f>SUM(B13:B14)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="99">
+      <c r="C15" s="100">
         <f>SUM(C13:C14)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="96">
+      <c r="D15" s="97">
         <f>SUM(D13:D14)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="100">
+      <c r="E15" s="101">
         <f>SUM(E13:E14)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="101">
+      <c r="F15" s="102">
         <f>SUM(F13:F14)</f>
         <v>0</v>
       </c>
@@ -1892,18 +1829,18 @@
       <c r="H15" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="I15" s="102">
+      <c r="I15" s="103">
         <f>SUM(I13:I14)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="98">
+      <c r="J15" s="99">
         <f>SUM(J13:J14)</f>
         <v>0</v>
       </c>
       <c r="K15" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L15" s="96">
+      <c r="L15" s="97">
         <f>SUM(L13:L14)</f>
         <v>0</v>
       </c>
@@ -1947,9 +1884,7 @@
       <c r="A17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="103">
-        <v>0</v>
-      </c>
+      <c r="B17" s="116"/>
       <c r="C17" s="10" t="s">
         <v>46</v>
       </c>
@@ -1979,14 +1914,12 @@
       <c r="A18">
         <v>1</v>
       </c>
-      <c r="B18" s="103">
-        <v>0</v>
-      </c>
+      <c r="B18" s="116"/>
       <c r="C18" s="15" t="str">
         <f>IF(B28&gt;B17,"Increase","Decrease")</f>
         <v>Decrease</v>
       </c>
-      <c r="D18" s="105">
+      <c r="D18" s="106">
         <f>B28-B17</f>
         <v>0</v>
       </c>
@@ -2014,9 +1947,7 @@
       <c r="A19">
         <v>2</v>
       </c>
-      <c r="B19" s="103">
-        <v>0</v>
-      </c>
+      <c r="B19" s="116"/>
       <c r="D19" s="10"/>
       <c r="E19" t="s">
         <v>50</v>
@@ -2057,9 +1988,7 @@
       <c r="A20">
         <v>3</v>
       </c>
-      <c r="B20" s="96">
-        <v>0</v>
-      </c>
+      <c r="B20" s="116"/>
       <c r="D20" s="10"/>
       <c r="E20" s="1"/>
       <c r="F20" s="10" t="s">
@@ -2074,7 +2003,7 @@
       <c r="I20" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="J20" s="104">
+      <c r="J20" s="105">
         <f>J15</f>
         <v>0</v>
       </c>
@@ -2082,7 +2011,7 @@
         <f>IF(J20 &gt;=L20, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L20" s="93">
+      <c r="L20" s="94">
         <f>L15</f>
         <v>0</v>
       </c>
@@ -2104,9 +2033,7 @@
       <c r="A21">
         <v>4</v>
       </c>
-      <c r="B21" s="96">
-        <v>0</v>
-      </c>
+      <c r="B21" s="116"/>
       <c r="D21" s="10"/>
       <c r="E21" s="1"/>
       <c r="F21" s="59" t="str">
@@ -2123,7 +2050,7 @@
       <c r="I21" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="J21" s="93">
+      <c r="J21" s="94">
         <f>D25</f>
         <v>0</v>
       </c>
@@ -2131,7 +2058,7 @@
         <f>IF(J21 =L21, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L21" s="93">
+      <c r="L21" s="94">
         <f>D25</f>
         <v>0</v>
       </c>
@@ -2153,10 +2080,7 @@
       <c r="A22">
         <v>5</v>
       </c>
-      <c r="B22" s="96">
-        <f t="shared" ref="B22" si="4">SUM(B17:B21)</f>
-        <v>0</v>
-      </c>
+      <c r="B22" s="116"/>
       <c r="D22" s="10"/>
       <c r="E22" s="1"/>
       <c r="F22" s="10" t="s">
@@ -2171,7 +2095,7 @@
       <c r="I22" s="56" t="s">
         <v>60</v>
       </c>
-      <c r="J22" s="104">
+      <c r="J22" s="105">
         <f>D26</f>
         <v>0</v>
       </c>
@@ -2179,7 +2103,7 @@
         <f>IF(J22 =L22, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L22" s="93">
+      <c r="L22" s="94">
         <f>D26</f>
         <v>0</v>
       </c>
@@ -2201,9 +2125,7 @@
       <c r="A23">
         <v>6</v>
       </c>
-      <c r="B23" s="103">
-        <v>0</v>
-      </c>
+      <c r="B23" s="116"/>
       <c r="D23" s="10"/>
       <c r="E23" s="38">
         <f>C2</f>
@@ -2223,7 +2145,7 @@
       <c r="I23" s="58" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="111">
+      <c r="J23" s="112">
         <f>SUM(J20:J22)</f>
         <v>0</v>
       </c>
@@ -2231,7 +2153,7 @@
         <f>IF(J23 =L23, "Paid", "Due")</f>
         <v>Paid</v>
       </c>
-      <c r="L23" s="93">
+      <c r="L23" s="94">
         <f>SUM(L20:L22)</f>
         <v>0</v>
       </c>
@@ -2253,9 +2175,7 @@
       <c r="A24">
         <v>7</v>
       </c>
-      <c r="B24" s="103">
-        <v>0</v>
-      </c>
+      <c r="B24" s="116"/>
       <c r="C24" s="15" t="s">
         <v>62</v>
       </c>
@@ -2287,24 +2207,22 @@
       <c r="A25">
         <v>8</v>
       </c>
-      <c r="B25" s="103">
-        <v>0</v>
-      </c>
+      <c r="B25" s="116"/>
       <c r="C25" s="2" t="str">
         <f>I21</f>
         <v>Mortgage</v>
       </c>
-      <c r="D25" s="103">
-        <v>0</v>
-      </c>
-      <c r="E25" s="87">
+      <c r="D25" s="104">
+        <v>0</v>
+      </c>
+      <c r="E25" s="88">
         <f>C$2</f>
         <v>0</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="106">
+      <c r="H25" s="107">
         <f>F2</f>
         <v>0</v>
       </c>
@@ -2338,33 +2256,31 @@
       <c r="A26">
         <v>9</v>
       </c>
-      <c r="B26" s="96">
-        <v>0</v>
-      </c>
+      <c r="B26" s="116"/>
       <c r="C26" s="2" t="str">
         <f>I22</f>
         <v>HOA</v>
       </c>
-      <c r="D26" s="103">
-        <v>0</v>
-      </c>
-      <c r="E26" s="87">
-        <f t="shared" ref="E26:E29" si="5">C$2</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="107">
+      <c r="D26" s="104">
+        <v>0</v>
+      </c>
+      <c r="E26" s="88">
+        <f t="shared" ref="E26:E29" si="4">C$2</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="108">
         <f>G2</f>
         <v>0</v>
       </c>
-      <c r="I26" s="98">
+      <c r="I26" s="99">
         <f>G17+C3+F2-I15-M50+E11</f>
         <v>0</v>
       </c>
-      <c r="J26" s="98">
+      <c r="J26" s="99">
         <f>G17+C3+C8+F2-M50</f>
         <v>0</v>
       </c>
-      <c r="K26" s="113">
+      <c r="K26" s="114">
         <v>5000</v>
       </c>
       <c r="L26" s="68" t="str">
@@ -2389,24 +2305,22 @@
       <c r="A27">
         <v>10</v>
       </c>
-      <c r="B27" s="96">
-        <v>0</v>
-      </c>
+      <c r="B27" s="116"/>
       <c r="C27" s="2" t="str">
         <f>B6</f>
         <v>Vacation Savings</v>
       </c>
-      <c r="D27" s="103">
-        <v>0</v>
-      </c>
-      <c r="E27" s="87">
-        <f t="shared" si="5"/>
+      <c r="D27" s="104">
+        <v>0</v>
+      </c>
+      <c r="E27" s="88">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G27" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="H27" s="108">
+      <c r="H27" s="109">
         <f>SUM(H25:H26)</f>
         <v>0</v>
       </c>
@@ -2432,25 +2346,22 @@
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="96">
-        <f t="shared" ref="B28" si="6">SUM(B23:B27)</f>
-        <v>0</v>
-      </c>
+      <c r="B28" s="116"/>
       <c r="C28" s="2" t="str">
         <f>B7</f>
         <v>Emergency Savings</v>
       </c>
-      <c r="D28" s="96">
-        <v>0</v>
-      </c>
-      <c r="E28" s="87">
-        <f t="shared" si="5"/>
+      <c r="D28" s="97">
+        <v>0</v>
+      </c>
+      <c r="E28" s="88">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="H28" s="109">
+      <c r="H28" s="110">
         <f>H27-D30</f>
         <v>0</v>
       </c>
@@ -2479,17 +2390,17 @@
         <f>B8</f>
         <v>Boost Savings</v>
       </c>
-      <c r="D29" s="96">
-        <v>0</v>
-      </c>
-      <c r="E29" s="87">
-        <f t="shared" si="5"/>
+      <c r="D29" s="97">
+        <v>0</v>
+      </c>
+      <c r="E29" s="88">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G29" t="s">
         <v>71</v>
       </c>
-      <c r="H29" s="110">
+      <c r="H29" s="111">
         <f>H27+G17</f>
         <v>0</v>
       </c>
@@ -2511,12 +2422,12 @@
       </c>
       <c r="Q29" s="30"/>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="B30" s="117"/>
+    <row r="30" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="87"/>
       <c r="C30" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="96">
+      <c r="D30" s="97">
         <f>SUM(D25:D29)</f>
         <v>0</v>
       </c>
@@ -2568,7 +2479,7 @@
       <c r="Q32" s="10"/>
       <c r="W32" s="10"/>
     </row>
-    <row r="33" spans="1:20" ht="52" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:20" ht="32" x14ac:dyDescent="0.2">
       <c r="B33" s="2" t="s">
         <v>72</v>
       </c>
@@ -2652,8 +2563,8 @@
       <c r="J35" s="76"/>
       <c r="K35" s="76"/>
       <c r="L35" s="76"/>
-      <c r="M35" s="104">
-        <f t="shared" ref="M35" si="7">SUM(C35:I35)</f>
+      <c r="M35" s="105">
+        <f t="shared" ref="M35" si="5">SUM(C35:I35)</f>
         <v>0</v>
       </c>
       <c r="N35" s="77">
@@ -2661,15 +2572,15 @@
         <v>0</v>
       </c>
       <c r="O35" s="77">
-        <f t="shared" ref="O35:O48" si="8">IFERROR(O34-M35/Q$50,0)</f>
+        <f t="shared" ref="O35:O48" si="6">IFERROR(O34-M35/Q$50,0)</f>
         <v>0</v>
       </c>
       <c r="P35" s="77">
-        <f t="shared" ref="P35:P48" si="9">IFERROR(P34-M35/Q$50,0)</f>
+        <f t="shared" ref="P35:P48" si="7">IFERROR(P34-M35/Q$50,0)</f>
         <v>0</v>
       </c>
       <c r="Q35" s="77">
-        <f t="shared" ref="Q35:Q48" si="10">IFERROR(Q34-M35/Q$50,0)</f>
+        <f t="shared" ref="Q35:Q48" si="8">IFERROR(Q34-M35/Q$50,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2691,24 +2602,24 @@
       <c r="J36" s="76"/>
       <c r="K36" s="76"/>
       <c r="L36" s="76"/>
-      <c r="M36" s="104">
+      <c r="M36" s="105">
         <f>SUM(C36:L36)</f>
         <v>0</v>
       </c>
       <c r="N36" s="77">
-        <f t="shared" ref="N36:N48" si="11">IFERROR(N35-M36/Q$50,0)</f>
+        <f t="shared" ref="N36:N48" si="9">IFERROR(N35-M36/Q$50,0)</f>
         <v>0</v>
       </c>
       <c r="O36" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P36" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q36" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P36" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q36" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -2730,24 +2641,24 @@
       <c r="J37" s="76"/>
       <c r="K37" s="76"/>
       <c r="L37" s="76"/>
-      <c r="M37" s="104">
+      <c r="M37" s="105">
         <f>SUM(C37:L37)</f>
         <v>0</v>
       </c>
       <c r="N37" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O37" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P37" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q37" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P37" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q37" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -2769,24 +2680,24 @@
       <c r="J38" s="76"/>
       <c r="K38" s="76"/>
       <c r="L38" s="76"/>
-      <c r="M38" s="104">
-        <f t="shared" ref="M38:M48" si="12">SUM(C38:L38)</f>
+      <c r="M38" s="105">
+        <f t="shared" ref="M38:M48" si="10">SUM(C38:L38)</f>
         <v>0</v>
       </c>
       <c r="N38" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O38" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P38" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q38" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P38" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q38" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -2808,24 +2719,24 @@
       <c r="J39" s="76"/>
       <c r="K39" s="76"/>
       <c r="L39" s="76"/>
-      <c r="M39" s="104">
-        <f t="shared" si="12"/>
+      <c r="M39" s="105">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N39" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O39" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P39" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q39" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P39" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q39" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -2847,24 +2758,24 @@
       <c r="J40" s="76"/>
       <c r="K40" s="76"/>
       <c r="L40" s="76"/>
-      <c r="M40" s="104">
-        <f t="shared" si="12"/>
+      <c r="M40" s="105">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N40" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O40" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P40" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q40" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P40" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q40" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -2886,24 +2797,24 @@
       <c r="J41" s="76"/>
       <c r="K41" s="76"/>
       <c r="L41" s="76"/>
-      <c r="M41" s="104">
+      <c r="M41" s="105">
         <f>SUM(C41:L41)</f>
         <v>0</v>
       </c>
       <c r="N41" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O41" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P41" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q41" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P41" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q41" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -2925,24 +2836,24 @@
       <c r="J42" s="76"/>
       <c r="K42" s="76"/>
       <c r="L42" s="76"/>
-      <c r="M42" s="104">
+      <c r="M42" s="105">
         <f>SUM(C42:L42)</f>
         <v>0</v>
       </c>
       <c r="N42" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O42" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P42" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q42" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P42" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q42" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -2964,24 +2875,24 @@
       <c r="J43" s="76"/>
       <c r="K43" s="76"/>
       <c r="L43" s="76"/>
-      <c r="M43" s="104">
-        <f t="shared" si="12"/>
+      <c r="M43" s="105">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N43" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O43" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P43" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q43" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P43" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q43" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -3003,24 +2914,24 @@
       <c r="J44" s="76"/>
       <c r="K44" s="76"/>
       <c r="L44" s="76"/>
-      <c r="M44" s="104">
-        <f t="shared" si="12"/>
+      <c r="M44" s="105">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N44" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O44" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P44" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q44" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P44" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q44" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -3042,24 +2953,24 @@
       <c r="J45" s="76"/>
       <c r="K45" s="76"/>
       <c r="L45" s="76"/>
-      <c r="M45" s="104">
-        <f t="shared" si="12"/>
+      <c r="M45" s="105">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N45" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O45" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P45" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q45" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P45" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q45" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -3081,24 +2992,24 @@
       <c r="J46" s="76"/>
       <c r="K46" s="76"/>
       <c r="L46" s="76"/>
-      <c r="M46" s="104">
-        <f t="shared" si="12"/>
+      <c r="M46" s="105">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N46" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O46" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P46" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q46" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P46" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q46" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -3120,24 +3031,24 @@
       <c r="J47" s="76"/>
       <c r="K47" s="76"/>
       <c r="L47" s="76"/>
-      <c r="M47" s="104">
-        <f t="shared" si="12"/>
+      <c r="M47" s="105">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N47" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O47" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P47" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q47" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P47" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q47" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -3159,24 +3070,24 @@
       <c r="J48" s="78"/>
       <c r="K48" s="78"/>
       <c r="L48" s="78"/>
-      <c r="M48" s="104">
-        <f t="shared" si="12"/>
+      <c r="M48" s="105">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N48" s="77">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O48" s="77">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P48" s="77">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q48" s="77">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P48" s="77">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Q48" s="77">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -3210,47 +3121,47 @@
       <c r="B50" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C50" s="103">
+      <c r="C50" s="104">
         <f>SUM(C35:C48)</f>
         <v>0</v>
       </c>
-      <c r="D50" s="103">
+      <c r="D50" s="104">
         <f>SUM(D35:D48)</f>
         <v>0</v>
       </c>
-      <c r="E50" s="103">
-        <f t="shared" ref="E50:L50" si="13">SUM(E36:E48)</f>
-        <v>0</v>
-      </c>
-      <c r="F50" s="103">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="G50" s="103">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="H50" s="103">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="I50" s="103">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J50" s="103">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="K50" s="103">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="L50" s="103">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="M50" s="103">
+      <c r="E50" s="104">
+        <f t="shared" ref="E50:L50" si="11">SUM(E36:E48)</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="104">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G50" s="104">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="H50" s="104">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="I50" s="104">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J50" s="104">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="K50" s="104">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="L50" s="104">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="M50" s="104">
         <f>SUM(M35:M48)</f>
         <v>0</v>
       </c>
@@ -3278,7 +3189,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:A9"/>
   </mergeCells>
-  <dataValidations count="47">
+  <dataValidations count="48">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{3170D0ED-69B8-2147-B2E8-C845548A1AEB}">
       <formula1>"Monday,Tuesday,Wednesday,Thursday,Friday,Saturday,Sunday"</formula1>
     </dataValidation>
@@ -3398,7 +3309,7 @@
       <formula1>0</formula1>
       <formula2>999999999.99</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Tank Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D25:D29 B17:B21 B23:B27" xr:uid="{DCEE984F-F387-8F43-B4D2-7C222E9FA32E}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Tank Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D25:D29" xr:uid="{DCEE984F-F387-8F43-B4D2-7C222E9FA32E}">
       <formula1>0</formula1>
       <formula2>999999999.99</formula2>
     </dataValidation>
@@ -3422,7 +3333,7 @@
       <formula1>0</formula1>
       <formula2>999999999.99</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Tank Total" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D30 B22 B28" xr:uid="{EB99C4F6-A363-7C40-A9E9-F2C68CD7797D}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Tank Total" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="D30" xr:uid="{EB99C4F6-A363-7C40-A9E9-F2C68CD7797D}">
       <formula1>0</formula1>
       <formula2>999999999.99</formula2>
     </dataValidation>
@@ -3466,12 +3377,16 @@
       <formula1>0</formula1>
       <formula2>999999999.99</formula2>
     </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Please enter a valid dollar amount." promptTitle="Dollar Amount" prompt="Please enter a dollar amount (e.g., 100.00, 250.50)" sqref="B17:B28" xr:uid="{4D60CF85-75C6-1448-A25A-EC8F9834344D}">
+      <formula1>0</formula1>
+      <formula2>999999999.99</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8812D7F7-4E2E-4C59-8640-33FA123A4EE8}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:W51"/>

</xml_diff>